<commit_message>
Add one-page Manager Summary tab to the webinar CEO plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGpsSZB9EZkEvXCwx9WBeN
</commit_message>
<xml_diff>
--- a/Zarthi_Webinar_CEO_Plan_22Sep26.xlsx
+++ b/Zarthi_Webinar_CEO_Plan_22Sep26.xlsx
@@ -6,26 +6,28 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="746" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Topics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Audience" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Funnel" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Offers" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Ads Plan" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Ad Copy" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Video Scripts" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Image Ideas" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Creatives" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="VSL Funnel" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Email &amp; WhatsApp" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Daily Plan" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Timeline" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Decisions" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Checklist" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Manager Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overview" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Topics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Audience" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Funnel" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Budget" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Offers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Ads Plan" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Ad Copy" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Video Scripts" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Image Ideas" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Creatives" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="VSL Funnel" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Email &amp; WhatsApp" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Daily Plan" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Timeline" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Decisions" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Checklist" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Checklist'!$A$3:$D$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Manager Summary'!$A$1:$E$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Checklist'!$A$3:$D$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,10 +38,10 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;₹&quot;#,##0"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="ddd dd-mmm"/>
+    <numFmt numFmtId="166" formatCode="ddd dd-mmm"/>
+    <numFmt numFmtId="167" formatCode="ddd d-mmm-yyyy"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -179,6 +181,24 @@
       <color rgb="FF0563C1"/>
       <sz val="10"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF262626"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1F6B3A"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="10">
@@ -371,7 +391,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -585,13 +605,13 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="20" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="20" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -600,12 +620,12 @@
     <xf numFmtId="9" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -615,6 +635,82 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="25" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -981,370 +1077,1907 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42.28515625" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" style="37" min="2" max="2"/>
-    <col width="59.85546875" customWidth="1" style="37" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="47" t="inlineStr">
-        <is>
-          <t>Topic</t>
+      <c r="A1" s="101" t="inlineStr">
+        <is>
+          <t>Zarthi Webinar Pilot: Plan Summary for Manager</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="47" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B2" s="47" t="inlineStr">
-        <is>
-          <t>Promise statement</t>
-        </is>
-      </c>
-      <c r="C2" s="54" t="n"/>
-      <c r="D2" s="54" t="n"/>
-      <c r="E2" s="54" t="n"/>
-      <c r="F2" s="54" t="n"/>
-      <c r="G2" s="54" t="n"/>
-      <c r="H2" s="55" t="n"/>
-    </row>
-    <row r="3" ht="23.25" customHeight="1">
-      <c r="A3" s="56" t="inlineStr">
-        <is>
-          <t>AI Is Eating Your Cloud Bill: How SRE &amp; DevOps Teams Cut Kubernetes and AI Costs</t>
-        </is>
-      </c>
-      <c r="B3" s="56" t="inlineStr">
-        <is>
-          <t>In 45 minutes, see the 5 places cloud money leaks in Kubernetes and AI workloads, and the fixes your team can ship this sprint, with a live teardown of real (anonymised) cloud bills.</t>
-        </is>
-      </c>
-      <c r="C3" s="54" t="n"/>
-      <c r="D3" s="54" t="n"/>
-      <c r="E3" s="54" t="n"/>
-      <c r="F3" s="54" t="n"/>
-      <c r="G3" s="54" t="n"/>
-      <c r="H3" s="55" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="34" t="n"/>
-      <c r="B4" s="53" t="inlineStr">
-        <is>
-          <t>Include</t>
-        </is>
-      </c>
-      <c r="C4" s="53" t="inlineStr">
-        <is>
-          <t>Exclude</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="35" t="inlineStr">
-        <is>
-          <t>Experience</t>
-        </is>
-      </c>
-      <c r="B5" s="56" t="inlineStr">
-        <is>
-          <t>3–15 years of total experience (pilot: wider net)</t>
-        </is>
-      </c>
-      <c r="C5" s="56" t="inlineStr">
-        <is>
-          <t>Freshers and students; job seekers</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30.75" customHeight="1">
-      <c r="A6" s="35" t="inlineStr">
-        <is>
-          <t>Seniority</t>
-        </is>
-      </c>
-      <c r="B6" s="56" t="inlineStr">
-        <is>
-          <t>SRE, DevOps, cloud, platform and backend engineers working on cloud, plus their leads and managers</t>
-        </is>
-      </c>
-      <c r="C6" s="56" t="inlineStr">
-        <is>
-          <t>C-suite (reached separately through direct outreach)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30.75" customHeight="1">
-      <c r="A7" s="35" t="inlineStr">
-        <is>
-          <t>Company type</t>
-        </is>
-      </c>
-      <c r="B7" s="50" t="inlineStr">
-        <is>
-          <t>Product and SaaS companies, GCCs, digital-first businesses (fintech, e-commerce, edtech, healthtech), in-house tech teams of enterprises (BFSI, healthcare, retail, manufacturing)</t>
-        </is>
-      </c>
-      <c r="C7" s="50" t="inlineStr">
-        <is>
-          <t>AWS partners and cloud MSPs (competitors). IT-services / outsourcing firms: CEO decision</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="35" t="inlineStr">
-        <is>
-          <t>Company size</t>
-        </is>
-      </c>
-      <c r="B8" s="50" t="inlineStr">
-        <is>
-          <t>50+ employees (existing MQL gate)</t>
-        </is>
-      </c>
-      <c r="C8" s="50" t="inlineStr">
-        <is>
-          <t>Under 50 employees</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="35" t="inlineStr">
-        <is>
-          <t>Geography</t>
-        </is>
-      </c>
-      <c r="B9" s="50" t="inlineStr">
-        <is>
-          <t>India: Bengaluru, Hyderabad, Pune, Delhi-NCR, Chennai, Mumbai</t>
-        </is>
-      </c>
-      <c r="C9" s="50" t="inlineStr">
-        <is>
-          <t>Outside India for this first episode</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="35" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="B10" s="50" t="inlineStr">
-        <is>
-          <t>Business email only</t>
-        </is>
-      </c>
-      <c r="C10" s="50" t="inlineStr">
-        <is>
-          <t>Gmail, Yahoo, Outlook and other personal domains</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="34" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="B12" s="53" t="inlineStr">
-        <is>
-          <t>How</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="35" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="B13" s="56" t="inlineStr">
-        <is>
-          <t>Job titles + 3–15 years + company size 51+. Lead Gen Form + CTO Thought Leader Ads. 60 registrations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30.75" customHeight="1">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="B14" s="56" t="inlineStr">
-        <is>
-          <t>Age 24–45. Cloud/DevOps interests, developer interests, Advantage+ broad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="35" t="inlineStr">
-        <is>
-          <t>Own channels</t>
-        </is>
-      </c>
-      <c r="B15" s="56" t="inlineStr">
-        <is>
-          <t>Not used for acquisition. Email + WhatsApp only after registration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="57" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="B16" s="58" t="inlineStr">
-        <is>
-          <t>Search (cost keywords) + Demand Gen (Discover, Gmail, YouTube feed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Funnel stage</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>Conservative</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="59" t="inlineStr">
+      <c r="A2" s="102" t="inlineStr">
+        <is>
+          <t>Numbers update automatically from the other tabs. Prepared by Shourya, 4-Oct-2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="103" t="inlineStr">
+        <is>
+          <t>1. Goal and key numbers</t>
+        </is>
+      </c>
+      <c r="B4" s="104" t="n"/>
+      <c r="C4" s="104" t="n"/>
+      <c r="D4" s="104" t="n"/>
+      <c r="E4" s="104" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="105" t="inlineStr">
         <is>
           <t>Live attendees (target)</t>
         </is>
       </c>
-      <c r="B18" s="60">
+      <c r="B5" s="106">
         <f>Funnel!B4</f>
         <v>200.0</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="46" t="inlineStr">
-        <is>
-          <t>TNC Landing Page Best Practices: Video Clips, Speaker USPs, Tracking, and Retargeting</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="43" t="inlineStr">
-        <is>
-          <t>Form Question in lead form : Need to discuss this----comapny mail id, name number</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="17" t="inlineStr">
-        <is>
-          <t>date and time</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>for eg : 29 oct Sat 11:00 AM</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="C5" s="64" t="n"/>
+      <c r="D5" s="64" t="n"/>
+      <c r="E5" s="65" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="105" t="inlineStr">
+        <is>
+          <t>Registrations needed (25% show-up + 10% buffer)</t>
+        </is>
+      </c>
+      <c r="B6" s="106">
+        <f>Funnel!B8</f>
+        <v>880.0</v>
+      </c>
+      <c r="C6" s="64" t="n"/>
+      <c r="D6" s="64" t="n"/>
+      <c r="E6" s="65" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="105" t="inlineStr">
+        <is>
+          <t>Ad budget (ex-GST)</t>
+        </is>
+      </c>
+      <c r="B7" s="107">
+        <f>Budget!F9</f>
+        <v>725000.0</v>
+      </c>
+      <c r="C7" s="64" t="n"/>
+      <c r="D7" s="64" t="n"/>
+      <c r="E7" s="65" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="105" t="inlineStr">
+        <is>
+          <t>Total budget (GST, Zoom, creatives, lucky draw)</t>
+        </is>
+      </c>
+      <c r="B8" s="107">
+        <f>Budget!F21</f>
+        <v>942690.0</v>
+      </c>
+      <c r="C8" s="64" t="n"/>
+      <c r="D8" s="64" t="n"/>
+      <c r="E8" s="65" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="105" t="inlineStr">
+        <is>
+          <t>Cost per live attendee</t>
+        </is>
+      </c>
+      <c r="B9" s="107">
+        <f>Budget!F23</f>
+        <v>4713.45</v>
+      </c>
+      <c r="C9" s="64" t="n"/>
+      <c r="D9" s="64" t="n"/>
+      <c r="E9" s="65" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="103" t="inlineStr">
+        <is>
+          <t>2. Webinar</t>
+        </is>
+      </c>
+      <c r="B11" s="104" t="n"/>
+      <c r="C11" s="104" t="n"/>
+      <c r="D11" s="104" t="n"/>
+      <c r="E11" s="104" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="108" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B12" s="109" t="inlineStr">
+        <is>
+          <t>AI Is Eating Your Cloud Bill: How SRE &amp; DevOps Teams Cut Kubernetes and AI Costs (Think Like a CTO, Episode 1)</t>
+        </is>
+      </c>
+      <c r="C12" s="64" t="n"/>
+      <c r="D12" s="64" t="n"/>
+      <c r="E12" s="65" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="108" t="inlineStr">
+        <is>
+          <t>Why this topic</t>
+        </is>
+      </c>
+      <c r="B13" s="109" t="inlineStr">
+        <is>
+          <t>Cloud waste rose to 29% in 2026 and managing AI cost is the #1 priority (State of FinOps 2026). Every SRE/DevOps engineer is blamed for the bill.</t>
+        </is>
+      </c>
+      <c r="C13" s="64" t="n"/>
+      <c r="D13" s="64" t="n"/>
+      <c r="E13" s="65" t="n"/>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="108" t="inlineStr">
+        <is>
+          <t>Date and time</t>
+        </is>
+      </c>
+      <c r="B14" s="109" t="inlineStr">
+        <is>
+          <t>Tue 27-Oct-2026, 4:00–5:00 PM IST (backup Wed 28-Oct). Zoom Webinars 500.</t>
+        </is>
+      </c>
+      <c r="C14" s="64" t="n"/>
+      <c r="D14" s="64" t="n"/>
+      <c r="E14" s="65" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="108" t="inlineStr">
+        <is>
+          <t>Speakers</t>
+        </is>
+      </c>
+      <c r="B15" s="109" t="inlineStr">
+        <is>
+          <t>CTO (15 years, ex-Microsoft) + CEO</t>
+        </is>
+      </c>
+      <c r="C15" s="64" t="n"/>
+      <c r="D15" s="64" t="n"/>
+      <c r="E15" s="65" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="108" t="inlineStr">
+        <is>
+          <t>Audience</t>
+        </is>
+      </c>
+      <c r="B16" s="109" t="inlineStr">
+        <is>
+          <t>SRE, DevOps, cloud and platform engineers and cloud developers; 3–15 years; Indian metros + tier-2 cities</t>
+        </is>
+      </c>
+      <c r="C16" s="64" t="n"/>
+      <c r="D16" s="64" t="n"/>
+      <c r="E16" s="65" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="108" t="inlineStr">
+        <is>
+          <t>How we find them</t>
+        </is>
+      </c>
+      <c r="B17" s="109" t="inlineStr">
+        <is>
+          <t>Paid ads on LinkedIn, Meta and Google only. Email + WhatsApp only after registration (reminders, follow-up).</t>
+        </is>
+      </c>
+      <c r="C17" s="64" t="n"/>
+      <c r="D17" s="64" t="n"/>
+      <c r="E17" s="65" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1"/>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="103" t="inlineStr">
+        <is>
+          <t>3. Budget by platform</t>
+        </is>
+      </c>
+      <c r="B19" s="104" t="n"/>
+      <c r="C19" s="104" t="n"/>
+      <c r="D19" s="104" t="n"/>
+      <c r="E19" s="104" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="110" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="B25" s="42" t="inlineStr">
-        <is>
-          <t>https://zoom.us/pricing</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="B26" s="58" t="inlineStr">
-        <is>
-          <t>Zoom Workplace Pro: INR 1,580 per user per month (host). For 200 live: Zoom Webinars 500, ₹11,610/month (Budget tab).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="40" t="inlineStr">
-        <is>
-          <t>Duration / Participants</t>
-        </is>
-      </c>
-      <c r="B27" s="61" t="inlineStr">
-        <is>
-          <t>Pro meetings hold 100; Webinars 500 holds 500 attendees</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Recording</t>
-        </is>
-      </c>
-      <c r="B28" s="41" t="inlineStr">
-        <is>
-          <t>Local &amp; 10 GB cloud (per license)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="41" t="inlineStr">
-        <is>
-          <t>Mail</t>
-        </is>
-      </c>
-      <c r="B29" s="37" t="inlineStr">
-        <is>
-          <t>Zoom Mail and Calendar in the Zoom app</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30.75" customHeight="1">
-      <c r="A30" s="41" t="inlineStr">
-        <is>
-          <t>Clips</t>
-        </is>
-      </c>
-      <c r="B30" s="37" t="inlineStr">
-        <is>
-          <t>Effortlessly create, edit, and share short videos. Stored clips are easily discoverable, boosting engagement / Unlimited</t>
+      <c r="B20" s="110" t="inlineStr">
+        <is>
+          <t>Registrations</t>
+        </is>
+      </c>
+      <c r="C20" s="110" t="inlineStr">
+        <is>
+          <t>Ad spend (ex-GST)</t>
+        </is>
+      </c>
+      <c r="D20" s="110" t="inlineStr">
+        <is>
+          <t>Cost per registration</t>
+        </is>
+      </c>
+      <c r="E20" s="110" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="108" t="inlineStr">
+        <is>
+          <t>Meta (FB + Instagram)</t>
+        </is>
+      </c>
+      <c r="B21" s="111">
+        <f>Budget!B4+Budget!B5</f>
+        <v>640.0</v>
+      </c>
+      <c r="C21" s="112">
+        <f>Budget!F4+Budget!F5</f>
+        <v>424000.0</v>
+      </c>
+      <c r="D21" s="112">
+        <f>IFERROR(C21/B21,0)</f>
+        <v>662.5</v>
+      </c>
+      <c r="E21" s="109" t="inlineStr">
+        <is>
+          <t>Volume: most registrations at ₹700 each</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="108" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="B22" s="111">
+        <f>Budget!B6</f>
+        <v>60.0</v>
+      </c>
+      <c r="C22" s="112">
+        <f>Budget!F6</f>
+        <v>150000.0</v>
+      </c>
+      <c r="D22" s="112">
+        <f>IFERROR(C22/B22,0)</f>
+        <v>2500.0</v>
+      </c>
+      <c r="E22" s="109" t="inlineStr">
+        <is>
+          <t>Senior reach: exact job titles, ₹2,500 each</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="108" t="inlineStr">
+        <is>
+          <t>Google (Search + Demand Gen)</t>
+        </is>
+      </c>
+      <c r="B23" s="111">
+        <f>Budget!B7+Budget!B8</f>
+        <v>180.0</v>
+      </c>
+      <c r="C23" s="112">
+        <f>Budget!F7+Budget!F8</f>
+        <v>151000.0</v>
+      </c>
+      <c r="D23" s="112">
+        <f>IFERROR(C23/B23,0)</f>
+        <v>838.8888888888889</v>
+      </c>
+      <c r="E23" s="109" t="inlineStr">
+        <is>
+          <t>Intent: people searching cloud cost topics</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="113" t="inlineStr">
+        <is>
+          <t>Total ads</t>
+        </is>
+      </c>
+      <c r="B24" s="114">
+        <f>SUM(B21:B23)</f>
+        <v>880.0</v>
+      </c>
+      <c r="C24" s="115">
+        <f>SUM(C21:C23)</f>
+        <v>725000.0</v>
+      </c>
+      <c r="D24" s="115">
+        <f>IFERROR(C24/B24,0)</f>
+        <v>823.8636363636364</v>
+      </c>
+      <c r="E24" s="116" t="inlineStr">
+        <is>
+          <t>+ GST, Zoom, creatives and lucky draw = total budget above</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1"/>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="103" t="inlineStr">
+        <is>
+          <t>4. When the ads run</t>
+        </is>
+      </c>
+      <c r="B26" s="104" t="n"/>
+      <c r="C26" s="104" t="n"/>
+      <c r="D26" s="104" t="n"/>
+      <c r="E26" s="104" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="110" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="B27" s="110" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="C27" s="110" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="D27" s="110" t="inlineStr">
+        <is>
+          <t>Ad budget</t>
+        </is>
+      </c>
+      <c r="E27" s="110" t="inlineStr">
+        <is>
+          <t>What happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="108" t="inlineStr">
+        <is>
+          <t>1. Test</t>
+        </is>
+      </c>
+      <c r="B28" s="117">
+        <f>Budget!B27</f>
+        <v>46304.0</v>
+      </c>
+      <c r="C28" s="117">
+        <f>Budget!C27</f>
+        <v>46308.0</v>
+      </c>
+      <c r="D28" s="112">
+        <f>Budget!F27</f>
+        <v>145000.0</v>
+      </c>
+      <c r="E28" s="109" t="inlineStr">
+        <is>
+          <t>Find the cheapest ads. CEO review on Tue 13-Oct before more money is released.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="108" t="inlineStr">
+        <is>
+          <t>2. Scale</t>
+        </is>
+      </c>
+      <c r="B29" s="117">
+        <f>Budget!B28</f>
+        <v>46309.0</v>
+      </c>
+      <c r="C29" s="117">
+        <f>Budget!C28</f>
+        <v>46318.0</v>
+      </c>
+      <c r="D29" s="112">
+        <f>Budget!F28</f>
+        <v>493000.00000000006</v>
+      </c>
+      <c r="E29" s="109" t="inlineStr">
+        <is>
+          <t>Money behind the winning ads only; retargeting on; new creatives every 4–5 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="108" t="inlineStr">
+        <is>
+          <t>3. Last call</t>
+        </is>
+      </c>
+      <c r="B30" s="117">
+        <f>Budget!B29</f>
+        <v>46319.0</v>
+      </c>
+      <c r="C30" s="117">
+        <f>Budget!C29</f>
+        <v>46321.0</v>
+      </c>
+      <c r="D30" s="112">
+        <f>Budget!F29</f>
+        <v>87000.0</v>
+      </c>
+      <c r="E30" s="109" t="inlineStr">
+        <is>
+          <t>Countdown ads. Ads stop the night before the webinar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="113" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B31" s="118">
+        <f>Budget!B27</f>
+        <v>46304.0</v>
+      </c>
+      <c r="C31" s="118">
+        <f>Budget!C29</f>
+        <v>46321.0</v>
+      </c>
+      <c r="D31" s="115">
+        <f>SUM(D28:D30)</f>
+        <v>725000.0</v>
+      </c>
+      <c r="E31" s="113" t="str">
+        <f>Budget!D30&amp;" days of ads"</f>
+        <v>18 days of ads</v>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1"/>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="103" t="inlineStr">
+        <is>
+          <t>5. Offers and creatives</t>
+        </is>
+      </c>
+      <c r="B33" s="104" t="n"/>
+      <c r="C33" s="104" t="n"/>
+      <c r="D33" s="104" t="n"/>
+      <c r="E33" s="104" t="n"/>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="108" t="inlineStr">
+        <is>
+          <t>When they register</t>
+        </is>
+      </c>
+      <c r="B34" s="109" t="inlineStr">
+        <is>
+          <t>Free 27-point Cloud &amp; Kubernetes Cost Leak Checklist (instant) + chance to get their own bill torn down live.</t>
+        </is>
+      </c>
+      <c r="C34" s="64" t="n"/>
+      <c r="D34" s="64" t="n"/>
+      <c r="E34" s="65" t="n"/>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="108" t="inlineStr">
+        <is>
+          <t>Only for live attendees</t>
+        </is>
+      </c>
+      <c r="B35" s="109" t="inlineStr">
+        <is>
+          <t>Full playbook, CTO-signed certificate, ₹20,000 lucky draw, 20 free Cloud Cost Reviews (sales pipeline).</t>
+        </is>
+      </c>
+      <c r="C35" s="64" t="n"/>
+      <c r="D35" s="64" t="n"/>
+      <c r="E35" s="65" t="n"/>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="108" t="inlineStr">
+        <is>
+          <t>Creatives</t>
+        </is>
+      </c>
+      <c r="B36" s="109" t="str">
+        <f>Creatives!B26&amp;". Scripts, ad copy and design briefs are in the file. Shoot: Mon 5 / Tue 6 Oct."</f>
+        <v>10 videos, 6 statics, 3 carousels, 1 LinkedIn document, 2 Google ad sets. Scripts, ad copy and design briefs are in the file. Shoot: Mon 5 / Tue 6 Oct.</v>
+      </c>
+      <c r="C36" s="64" t="n"/>
+      <c r="D36" s="64" t="n"/>
+      <c r="E36" s="65" t="n"/>
+    </row>
+    <row r="37" ht="30" customHeight="1"/>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="103" t="inlineStr">
+        <is>
+          <t>6. Realistic outcome</t>
+        </is>
+      </c>
+      <c r="B38" s="104" t="n"/>
+      <c r="C38" s="104" t="n"/>
+      <c r="D38" s="104" t="n"/>
+      <c r="E38" s="104" t="n"/>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="110" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B39" s="110" t="inlineStr">
+        <is>
+          <t>Live attendees</t>
+        </is>
+      </c>
+      <c r="C39" s="110" t="inlineStr"/>
+      <c r="D39" s="110" t="inlineStr"/>
+      <c r="E39" s="110" t="inlineStr">
+        <is>
+          <t>What drives it</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="108" t="inlineStr">
+        <is>
+          <t>Worst case</t>
+        </is>
+      </c>
+      <c r="B40" s="119" t="inlineStr">
+        <is>
+          <t>70–100</t>
+        </is>
+      </c>
+      <c r="C40" s="64" t="n"/>
+      <c r="D40" s="65" t="n"/>
+      <c r="E40" s="109" t="inlineStr">
+        <is>
+          <t>Cost per registration above ₹1,000 and show-up near 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="105" t="inlineStr">
+        <is>
+          <t>Most likely</t>
+        </is>
+      </c>
+      <c r="B41" s="120" t="inlineStr">
+        <is>
+          <t>120–160</t>
+        </is>
+      </c>
+      <c r="C41" s="64" t="n"/>
+      <c r="D41" s="65" t="n"/>
+      <c r="E41" s="121" t="inlineStr">
+        <is>
+          <t>Cost near ₹700–850 per registration, show-up 22–28%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="108" t="inlineStr">
+        <is>
+          <t>Best case</t>
+        </is>
+      </c>
+      <c r="B42" s="119" t="inlineStr">
+        <is>
+          <t>200+</t>
+        </is>
+      </c>
+      <c r="C42" s="64" t="n"/>
+      <c r="D42" s="65" t="n"/>
+      <c r="E42" s="109" t="inlineStr">
+        <is>
+          <t>Winning video found in test week, cost ≤ ₹700, show-up 30%+</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="108" t="inlineStr">
+        <is>
+          <t>Biggest lever</t>
+        </is>
+      </c>
+      <c r="B43" s="109" t="inlineStr">
+        <is>
+          <t>Show-up rate. Moving from 25% to 30% cuts registrations needed from 880 to ~733 and saves about ₹1.4 lakh.</t>
+        </is>
+      </c>
+      <c r="C43" s="64" t="n"/>
+      <c r="D43" s="64" t="n"/>
+      <c r="E43" s="65" t="n"/>
+    </row>
+    <row r="44" ht="30" customHeight="1"/>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="103" t="inlineStr">
+        <is>
+          <t>7. Decisions needed</t>
+        </is>
+      </c>
+      <c r="B45" s="104" t="n"/>
+      <c r="C45" s="104" t="n"/>
+      <c r="D45" s="104" t="n"/>
+      <c r="E45" s="104" t="n"/>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="122" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B46" s="109" t="inlineStr">
+        <is>
+          <t>Approve the topic and the date (Tue 27-Oct, 4 PM)</t>
+        </is>
+      </c>
+      <c r="C46" s="64" t="n"/>
+      <c r="D46" s="64" t="n"/>
+      <c r="E46" s="65" t="n"/>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="122" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B47" s="109" t="str">
+        <f>"Approve the total budget of ₹"&amp;TEXT(Budget!F21,"#,##0")&amp;", released in 3 stages"</f>
+        <v>Approve the total budget of ₹942,690, released in 3 stages</v>
+      </c>
+      <c r="C47" s="64" t="n"/>
+      <c r="D47" s="64" t="n"/>
+      <c r="E47" s="65" t="n"/>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="122" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B48" s="109" t="inlineStr">
+        <is>
+          <t>Approve Zoom Webinars 500 (₹11,610/month), needed for 200+ live</t>
+        </is>
+      </c>
+      <c r="C48" s="64" t="n"/>
+      <c r="D48" s="64" t="n"/>
+      <c r="E48" s="65" t="n"/>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="122" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B49" s="109" t="inlineStr">
+        <is>
+          <t>Approve the offers and the ₹20,000 lucky draw</t>
+        </is>
+      </c>
+      <c r="C49" s="64" t="n"/>
+      <c r="D49" s="64" t="n"/>
+      <c r="E49" s="65" t="n"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="122" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B50" s="109" t="str">
+        <f>"Approve creative production (₹"&amp;TEXT(Creatives!F41,"#,##0")&amp;") and a 2-hour CEO + CTO shoot on 5–6 Oct"</f>
+        <v>Approve creative production (₹44,000) and a 2-hour CEO + CTO shoot on 5–6 Oct</v>
+      </c>
+      <c r="C50" s="64" t="n"/>
+      <c r="D50" s="64" t="n"/>
+      <c r="E50" s="65" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="122" t="inlineStr">
+        <is>
+          <t>6.</t>
+        </is>
+      </c>
+      <c r="B51" s="109" t="inlineStr">
+        <is>
+          <t>Agree the commitment: target 200 live, commit 120–150, review on 13-Oct</t>
+        </is>
+      </c>
+      <c r="C51" s="64" t="n"/>
+      <c r="D51" s="64" t="n"/>
+      <c r="E51" s="65" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="102" t="inlineStr">
+        <is>
+          <t>Details: Budget, Ads Plan, Ad Copy, Video Scripts, Image Ideas, Offers, Daily Plan, Timeline and Decisions tabs.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B2:H2"/>
+  <mergeCells count="24">
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B34:E34"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="62" t="inlineStr">
+        <is>
+          <t>Video scripts: every video, scene by scene</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="74" t="inlineStr">
+        <is>
+          <t>One 2-hour shoot (Mon 5 or Tue 6 Oct) covers V1–V4, V6 and V8. Add burned-in captions to every video. [CTO name] = replace with the real name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="63" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="B3" s="63" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C3" s="63" t="inlineStr">
+        <is>
+          <t>Shot / visual</t>
+        </is>
+      </c>
+      <c r="D3" s="63" t="inlineStr">
+        <is>
+          <t>Voiceover (exact words)</t>
+        </is>
+      </c>
+      <c r="E3" s="63" t="inlineStr">
+        <is>
+          <t>On-screen text</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="95" t="inlineStr">
+        <is>
+          <t>V1: Main VSL, 3–3.5 min, 16:9 (landing page)</t>
+        </is>
+      </c>
+      <c r="B4" s="95" t="n"/>
+      <c r="C4" s="95" t="n"/>
+      <c r="D4" s="95" t="n"/>
+      <c r="E4" s="95" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="67" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B5" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:10</t>
+        </is>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>CTO close-up, office background. Cut-in: a monthly cost graph rising.</t>
+        </is>
+      </c>
+      <c r="D5" s="66" t="inlineStr">
+        <is>
+          <t>Your cloud bill went up again this month. Traffic didn't. Somewhere in your clusters, money is leaking, and in most teams nobody owns finding it.</t>
+        </is>
+      </c>
+      <c r="E5" s="66" t="inlineStr">
+        <is>
+          <t>Bill ↑. Traffic →. (example)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B6" s="66" t="inlineStr">
+        <is>
+          <t>0:10–0:35</t>
+        </is>
+      </c>
+      <c r="C6" s="66" t="inlineStr">
+        <is>
+          <t>B-roll: Kubernetes dashboard, GPU usage graph, Slack message 'why is AWS so high?'</t>
+        </is>
+      </c>
+      <c r="D6" s="66" t="inlineStr">
+        <is>
+          <t>In 2026 it's getting worse. AI workloads, GPUs, idle dev clusters, oversized nodes. The State of FinOps report found 29% of cloud spend is wasted, and it went up for the first time in five years. And when finance asks why, they don't ask the vendor. They ask the SRE and DevOps team.</t>
+        </is>
+      </c>
+      <c r="E6" s="66" t="inlineStr">
+        <is>
+          <t>29% of cloud spend is wasted (State of FinOps 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="inlineStr">
+        <is>
+          <t>0:35–1:05</t>
+        </is>
+      </c>
+      <c r="C7" s="66" t="inlineStr">
+        <is>
+          <t>CTO introduces himself; quick cut to CEO.</t>
+        </is>
+      </c>
+      <c r="D7" s="66" t="inlineStr">
+        <is>
+          <t>I'm [CTO name], CTO at Zarthi. I've spent 15 years building cloud platforms, including at Microsoft. My team reviews cloud setups for Indian product companies every week, and the same five leaks show up almost every time. CEO: That's why we started Think Like a CTO: free sessions for engineers who want to make the calls, not just close the tickets.</t>
+        </is>
+      </c>
+      <c r="E7" s="66" t="inlineStr">
+        <is>
+          <t>[CTO name] · CTO, Zarthi · ex-Microsoft</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="67" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B8" s="66" t="inlineStr">
+        <is>
+          <t>1:05–1:50</t>
+        </is>
+      </c>
+      <c r="C8" s="66" t="inlineStr">
+        <is>
+          <t>Screen recording: 'kubectl top pods' next to the requests in a deployment YAML; requests highlighted in red.</t>
+        </is>
+      </c>
+      <c r="D8" s="66" t="inlineStr">
+        <is>
+          <t>Let me give you leak number one right now. Idle and oversized compute. Pull the CPU and memory requests for your top ten workloads and compare them with what they actually use. If requests are double the usage, you're paying for air. Fix it with rightsizing and autoscaling. That's one of five.</t>
+        </is>
+      </c>
+      <c r="E8" s="66" t="inlineStr">
+        <is>
+          <t>Leak #1: requests ≫ usage = paying for air</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="67" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B9" s="66" t="inlineStr">
+        <is>
+          <t>1:50–2:30</t>
+        </is>
+      </c>
+      <c r="C9" s="66" t="inlineStr">
+        <is>
+          <t>CTO on camera; graphics pop in for each benefit.</t>
+        </is>
+      </c>
+      <c r="D9" s="66" t="inlineStr">
+        <is>
+          <t>On Tuesday, 27 October at 4 PM, I'll walk through all five leaks, including GPU and AI inference costs, and tear down real, anonymised cloud bills that you send in. You get the 27-point Cost Leak Checklist the moment you register. Join live and you also get the full playbook, a certificate, and a chance to win vouchers. The first 300 people also get our AI Cost Guardrails Pack.</t>
+        </is>
+      </c>
+      <c r="E9" s="66" t="inlineStr">
+        <is>
+          <t>Free checklist now · Playbook + certificate + lucky draw live</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="67" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B10" s="66" t="inlineStr">
+        <is>
+          <t>2:30–2:55</t>
+        </is>
+      </c>
+      <c r="C10" s="66" t="inlineStr">
+        <is>
+          <t>CTO, two-column 'For / Not for' graphic.</t>
+        </is>
+      </c>
+      <c r="D10" s="66" t="inlineStr">
+        <is>
+          <t>This is for SREs, DevOps, platform and cloud engineers, and developers who run things on AWS, Azure or GCP. It's not a beginner course, and it's not a sales pitch. There's no product demo.</t>
+        </is>
+      </c>
+      <c r="E10" s="66" t="inlineStr">
+        <is>
+          <t>For: SRE · DevOps · Platform · Cloud · Developers</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="67" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B11" s="66" t="inlineStr">
+        <is>
+          <t>2:55–3:20</t>
+        </is>
+      </c>
+      <c r="C11" s="66" t="inlineStr">
+        <is>
+          <t>CTO points down; date card; form appears below the video.</t>
+        </is>
+      </c>
+      <c r="D11" s="66" t="inlineStr">
+        <is>
+          <t>Forty-five minutes. Free. Register below, and add your cloud bill question in the form. If yours is picked, we tear it down live. See you on the 27th.</t>
+        </is>
+      </c>
+      <c r="E11" s="66" t="inlineStr">
+        <is>
+          <t>Tue 27 Oct · 4 PM IST · Free · Register below ↓</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="95" t="inlineStr">
+        <is>
+          <t>V2: 60-second cut, 16:9 / 1:1 / 9:16 (Google Demand Gen, LinkedIn, Meta)</t>
+        </is>
+      </c>
+      <c r="B12" s="95" t="n"/>
+      <c r="C12" s="95" t="n"/>
+      <c r="D12" s="95" t="n"/>
+      <c r="E12" s="95" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="67" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="B13" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:05</t>
+        </is>
+      </c>
+      <c r="C13" s="66" t="inlineStr">
+        <is>
+          <t>CTO close-up, bold caption.</t>
+        </is>
+      </c>
+      <c r="D13" s="66" t="inlineStr">
+        <is>
+          <t>29% of cloud spend is wasted. Here's where it hides in Kubernetes.</t>
+        </is>
+      </c>
+      <c r="E13" s="66" t="inlineStr">
+        <is>
+          <t>29% wasted</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="67" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="B14" s="66" t="inlineStr">
+        <is>
+          <t>0:05–0:20</t>
+        </is>
+      </c>
+      <c r="C14" s="66" t="inlineStr">
+        <is>
+          <t>B-roll of dashboards; CTO voice.</t>
+        </is>
+      </c>
+      <c r="D14" s="66" t="inlineStr">
+        <is>
+          <t>Idle dev clusters. Pods asking for twice the CPU they use. GPUs sitting at 10%. And the bill lands on the SRE and DevOps team.</t>
+        </is>
+      </c>
+      <c r="E14" s="66" t="inlineStr">
+        <is>
+          <t>Idle clusters · Oversized pods · Idle GPUs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="67" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="B15" s="66" t="inlineStr">
+        <is>
+          <t>0:20–0:40</t>
+        </is>
+      </c>
+      <c r="C15" s="66" t="inlineStr">
+        <is>
+          <t>Screen: kubectl top vs YAML requests.</t>
+        </is>
+      </c>
+      <c r="D15" s="66" t="inlineStr">
+        <is>
+          <t>Quick check: compare requests with real usage for your top ten workloads. Double? You're paying for air.</t>
+        </is>
+      </c>
+      <c r="E15" s="66" t="inlineStr">
+        <is>
+          <t>Requests vs usage: check yours</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="67" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="B16" s="66" t="inlineStr">
+        <is>
+          <t>0:40–0:55</t>
+        </is>
+      </c>
+      <c r="C16" s="66" t="inlineStr">
+        <is>
+          <t>CTO; benefit graphics.</t>
+        </is>
+      </c>
+      <c r="D16" s="66" t="inlineStr">
+        <is>
+          <t>On 27 October I'll show all five leaks and tear down real bills live. Register and get our 27-point Cost Leak Checklist free.</t>
+        </is>
+      </c>
+      <c r="E16" s="66" t="inlineStr">
+        <is>
+          <t>Free checklist on sign-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="67" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="B17" s="66" t="inlineStr">
+        <is>
+          <t>0:55–1:00</t>
+        </is>
+      </c>
+      <c r="C17" s="66" t="inlineStr">
+        <is>
+          <t>End card with date and button.</t>
+        </is>
+      </c>
+      <c r="D17" s="66" t="inlineStr">
+        <is>
+          <t>Free, 45 minutes. Link below.</t>
+        </is>
+      </c>
+      <c r="E17" s="66" t="inlineStr">
+        <is>
+          <t>Tue 27 Oct · 4 PM · Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="95" t="inlineStr">
+        <is>
+          <t>V3: CTO talking head, 30 s, 9:16 + 4:5 (Meta, LinkedIn)</t>
+        </is>
+      </c>
+      <c r="B18" s="95" t="n"/>
+      <c r="C18" s="95" t="n"/>
+      <c r="D18" s="95" t="n"/>
+      <c r="E18" s="95" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="67" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="B19" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:03</t>
+        </is>
+      </c>
+      <c r="C19" s="66" t="inlineStr">
+        <is>
+          <t>CTO, phone camera, eye level.</t>
+        </is>
+      </c>
+      <c r="D19" s="66" t="inlineStr">
+        <is>
+          <t>Three places your Kubernetes bill leaks. Number two surprises everyone.</t>
+        </is>
+      </c>
+      <c r="E19" s="66" t="inlineStr">
+        <is>
+          <t>3 Kubernetes bill leaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="67" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="B20" s="66" t="inlineStr">
+        <is>
+          <t>0:03–0:12</t>
+        </is>
+      </c>
+      <c r="C20" s="66" t="inlineStr">
+        <is>
+          <t>CTO counts on fingers.</t>
+        </is>
+      </c>
+      <c r="D20" s="66" t="inlineStr">
+        <is>
+          <t>One: pods asking for far more CPU than they use. Two: logs. Teams spend more storing debug logs than running the app.</t>
+        </is>
+      </c>
+      <c r="E20" s="66" t="inlineStr">
+        <is>
+          <t>1. Oversized pods  2. Log storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="B21" s="66" t="inlineStr">
+        <is>
+          <t>0:12–0:22</t>
+        </is>
+      </c>
+      <c r="C21" s="66" t="inlineStr">
+        <is>
+          <t>CTO.</t>
+        </is>
+      </c>
+      <c r="D21" s="66" t="inlineStr">
+        <is>
+          <t>Three: dev and staging clusters running all night and every weekend.</t>
+        </is>
+      </c>
+      <c r="E21" s="66" t="inlineStr">
+        <is>
+          <t>3. Clusters that never sleep</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="67" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="B22" s="66" t="inlineStr">
+        <is>
+          <t>0:22–0:30</t>
+        </is>
+      </c>
+      <c r="C22" s="66" t="inlineStr">
+        <is>
+          <t>CTO points to caption.</t>
+        </is>
+      </c>
+      <c r="D22" s="66" t="inlineStr">
+        <is>
+          <t>I'll show the other two, and the fixes, live on the 27th. Free. Link below.</t>
+        </is>
+      </c>
+      <c r="E22" s="66" t="inlineStr">
+        <is>
+          <t>Free live session · 27 Oct · 4 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="95" t="inlineStr">
+        <is>
+          <t>V4: CEO talking head, 30 s, 4:5 + 1:1 (Meta, LinkedIn)</t>
+        </is>
+      </c>
+      <c r="B23" s="95" t="n"/>
+      <c r="C23" s="95" t="n"/>
+      <c r="D23" s="95" t="n"/>
+      <c r="E23" s="95" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="67" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="B24" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:04</t>
+        </is>
+      </c>
+      <c r="C24" s="66" t="inlineStr">
+        <is>
+          <t>CEO, office.</t>
+        </is>
+      </c>
+      <c r="D24" s="66" t="inlineStr">
+        <is>
+          <t>The engineers who get promoted fastest can explain the cloud bill.</t>
+        </is>
+      </c>
+      <c r="E24" s="66" t="inlineStr">
+        <is>
+          <t>Can you explain your cloud bill?</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="67" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="B25" s="66" t="inlineStr">
+        <is>
+          <t>0:04–0:18</t>
+        </is>
+      </c>
+      <c r="C25" s="66" t="inlineStr">
+        <is>
+          <t>CEO.</t>
+        </is>
+      </c>
+      <c r="D25" s="66" t="inlineStr">
+        <is>
+          <t>Not because they're accountants. Because when the bill jumps, the CTO needs someone who knows which service, which team, and which fix. That person gets trusted with bigger decisions.</t>
+        </is>
+      </c>
+      <c r="E25" s="66" t="inlineStr">
+        <is>
+          <t>Cost = a leadership skill</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="67" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="B26" s="66" t="inlineStr">
+        <is>
+          <t>0:18–0:30</t>
+        </is>
+      </c>
+      <c r="C26" s="66" t="inlineStr">
+        <is>
+          <t>CEO; date card.</t>
+        </is>
+      </c>
+      <c r="D26" s="66" t="inlineStr">
+        <is>
+          <t>Our CTO is teaching exactly that, free, on 27 October. SREs, DevOps and cloud engineers: register below.</t>
+        </is>
+      </c>
+      <c r="E26" s="66" t="inlineStr">
+        <is>
+          <t>Free · 27 Oct · 4 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="95" t="inlineStr">
+        <is>
+          <t>V5: Myth vs fact reel, 15 s, 9:16 (Meta Reels/Stories)</t>
+        </is>
+      </c>
+      <c r="B27" s="95" t="n"/>
+      <c r="C27" s="95" t="n"/>
+      <c r="D27" s="95" t="n"/>
+      <c r="E27" s="95" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="67" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="B28" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:04</t>
+        </is>
+      </c>
+      <c r="C28" s="66" t="inlineStr">
+        <is>
+          <t>Big text on a dark background, beat-synced.</t>
+        </is>
+      </c>
+      <c r="D28" s="66" t="inlineStr">
+        <is>
+          <t>(music only)</t>
+        </is>
+      </c>
+      <c r="E28" s="66" t="inlineStr">
+        <is>
+          <t>MYTH: Autoscaling saves money.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="67" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="B29" s="66" t="inlineStr">
+        <is>
+          <t>0:04–0:09</t>
+        </is>
+      </c>
+      <c r="C29" s="66" t="inlineStr">
+        <is>
+          <t>Text card + screenshot of a node pool.</t>
+        </is>
+      </c>
+      <c r="D29" s="66" t="inlineStr">
+        <is>
+          <t>(music only)</t>
+        </is>
+      </c>
+      <c r="E29" s="66" t="inlineStr">
+        <is>
+          <t>FACT: Autoscaling on oversized requests scales the waste too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="67" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="B30" s="66" t="inlineStr">
+        <is>
+          <t>0:09–0:15</t>
+        </is>
+      </c>
+      <c r="C30" s="66" t="inlineStr">
+        <is>
+          <t>Speaker faces + date.</t>
+        </is>
+      </c>
+      <c r="D30" s="66" t="inlineStr">
+        <is>
+          <t>(music only)</t>
+        </is>
+      </c>
+      <c r="E30" s="66" t="inlineStr">
+        <is>
+          <t>5 leaks + live bill teardown · Free · 27 Oct · Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="95" t="inlineStr">
+        <is>
+          <t>V6: Whiteboard explainer, 45 s, 9:16 + 16:9</t>
+        </is>
+      </c>
+      <c r="B31" s="95" t="n"/>
+      <c r="C31" s="95" t="n"/>
+      <c r="D31" s="95" t="n"/>
+      <c r="E31" s="95" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="67" t="inlineStr">
+        <is>
+          <t>V6</t>
+        </is>
+      </c>
+      <c r="B32" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:05</t>
+        </is>
+      </c>
+      <c r="C32" s="66" t="inlineStr">
+        <is>
+          <t>CTO at a whiteboard, writes ₹100.</t>
+        </is>
+      </c>
+      <c r="D32" s="66" t="inlineStr">
+        <is>
+          <t>Follow 100 rupees of cloud spend and watch 29 disappear.</t>
+        </is>
+      </c>
+      <c r="E32" s="66" t="inlineStr">
+        <is>
+          <t>Where does ₹100 go?</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="67" t="inlineStr">
+        <is>
+          <t>V6</t>
+        </is>
+      </c>
+      <c r="B33" s="66" t="inlineStr">
+        <is>
+          <t>0:05–0:30</t>
+        </is>
+      </c>
+      <c r="C33" s="66" t="inlineStr">
+        <is>
+          <t>CTO draws boxes: compute, storage, data transfer, AI/GPU; crosses out parts.</t>
+        </is>
+      </c>
+      <c r="D33" s="66" t="inlineStr">
+        <is>
+          <t>Compute you reserved but don't use. Storage nobody deleted. Data moving between zones for no reason. GPUs waiting for jobs. Add it up: about 29 rupees of every 100.</t>
+        </is>
+      </c>
+      <c r="E33" s="66" t="inlineStr">
+        <is>
+          <t>Unused compute · Old storage · Cross-zone traffic · Idle GPUs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="67" t="inlineStr">
+        <is>
+          <t>V6</t>
+        </is>
+      </c>
+      <c r="B34" s="66" t="inlineStr">
+        <is>
+          <t>0:30–0:45</t>
+        </is>
+      </c>
+      <c r="C34" s="66" t="inlineStr">
+        <is>
+          <t>CTO caps the marker.</t>
+        </is>
+      </c>
+      <c r="D34" s="66" t="inlineStr">
+        <is>
+          <t>On 27 October I'll show how to find each one in your own account, and fix it. Free. Register below.</t>
+        </is>
+      </c>
+      <c r="E34" s="66" t="inlineStr">
+        <is>
+          <t>Free · 27 Oct · 4 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="95" t="inlineStr">
+        <is>
+          <t>V7: Engineer POV, 25 s, 9:16 (Meta Reels). Use only if the story is true; change the numbers to the real ones.</t>
+        </is>
+      </c>
+      <c r="B35" s="95" t="n"/>
+      <c r="C35" s="95" t="n"/>
+      <c r="D35" s="95" t="n"/>
+      <c r="E35" s="95" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="67" t="inlineStr">
+        <is>
+          <t>V7</t>
+        </is>
+      </c>
+      <c r="B36" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:04</t>
+        </is>
+      </c>
+      <c r="C36" s="66" t="inlineStr">
+        <is>
+          <t>Zarthi engineer, selfie, natural light.</t>
+        </is>
+      </c>
+      <c r="D36" s="66" t="inlineStr">
+        <is>
+          <t>Our staging clusters ran all night. Nobody used them after 8 PM.</t>
+        </is>
+      </c>
+      <c r="E36" s="66" t="inlineStr">
+        <is>
+          <t>Staging, running 24/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="67" t="inlineStr">
+        <is>
+          <t>V7</t>
+        </is>
+      </c>
+      <c r="B37" s="66" t="inlineStr">
+        <is>
+          <t>0:04–0:16</t>
+        </is>
+      </c>
+      <c r="C37" s="66" t="inlineStr">
+        <is>
+          <t>Engineer; screen of a cron schedule.</t>
+        </is>
+      </c>
+      <c r="D37" s="66" t="inlineStr">
+        <is>
+          <t>One scheduled scale-down at night and on weekends. Our staging bill dropped by about a third the next month.</t>
+        </is>
+      </c>
+      <c r="E37" s="66" t="inlineStr">
+        <is>
+          <t>1 schedule → staging bill ↓ (use real number)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="67" t="inlineStr">
+        <is>
+          <t>V7</t>
+        </is>
+      </c>
+      <c r="B38" s="66" t="inlineStr">
+        <is>
+          <t>0:16–0:25</t>
+        </is>
+      </c>
+      <c r="C38" s="66" t="inlineStr">
+        <is>
+          <t>Engineer.</t>
+        </is>
+      </c>
+      <c r="D38" s="66" t="inlineStr">
+        <is>
+          <t>Our CTO is sharing five fixes like this live on the 27th. It's free. Link below.</t>
+        </is>
+      </c>
+      <c r="E38" s="66" t="inlineStr">
+        <is>
+          <t>Free live session · 27 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="95" t="inlineStr">
+        <is>
+          <t>V8: CEO + CTO podcast clip, 40 s, 1:1 + 9:16</t>
+        </is>
+      </c>
+      <c r="B39" s="95" t="n"/>
+      <c r="C39" s="95" t="n"/>
+      <c r="D39" s="95" t="n"/>
+      <c r="E39" s="95" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="67" t="inlineStr">
+        <is>
+          <t>V8</t>
+        </is>
+      </c>
+      <c r="B40" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:05</t>
+        </is>
+      </c>
+      <c r="C40" s="66" t="inlineStr">
+        <is>
+          <t>Two-shot, mics visible.</t>
+        </is>
+      </c>
+      <c r="D40" s="66" t="inlineStr">
+        <is>
+          <t>CEO: Who owns the cloud bill in most teams?</t>
+        </is>
+      </c>
+      <c r="E40" s="66" t="inlineStr">
+        <is>
+          <t>Who owns the cloud bill?</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="67" t="inlineStr">
+        <is>
+          <t>V8</t>
+        </is>
+      </c>
+      <c r="B41" s="66" t="inlineStr">
+        <is>
+          <t>0:05–0:25</t>
+        </is>
+      </c>
+      <c r="C41" s="66" t="inlineStr">
+        <is>
+          <t>Close-up CTO.</t>
+        </is>
+      </c>
+      <c r="D41" s="66" t="inlineStr">
+        <is>
+          <t>CTO: Honestly? Nobody, until it doubles. Then it's suddenly the DevOps team's problem. The fix isn't a tool. It's making cost visible per team, with guardrails so nobody can launch a 64-core pod by accident.</t>
+        </is>
+      </c>
+      <c r="E41" s="66" t="inlineStr">
+        <is>
+          <t>Make cost visible · Add guardrails</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="67" t="inlineStr">
+        <is>
+          <t>V8</t>
+        </is>
+      </c>
+      <c r="B42" s="66" t="inlineStr">
+        <is>
+          <t>0:25–0:40</t>
+        </is>
+      </c>
+      <c r="C42" s="66" t="inlineStr">
+        <is>
+          <t>Two-shot, date card.</t>
+        </is>
+      </c>
+      <c r="D42" s="66" t="inlineStr">
+        <is>
+          <t>CEO: We're going deep on this live on the 27th. CTO: Bring your bill. We'll tear it down.</t>
+        </is>
+      </c>
+      <c r="E42" s="66" t="inlineStr">
+        <is>
+          <t>Free · 27 Oct · 4 PM IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="95" t="inlineStr">
+        <is>
+          <t>V9: Bumper, 6 s, 16:9 (Google Demand Gen video)</t>
+        </is>
+      </c>
+      <c r="B43" s="95" t="n"/>
+      <c r="C43" s="95" t="n"/>
+      <c r="D43" s="95" t="n"/>
+      <c r="E43" s="95" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="67" t="inlineStr">
+        <is>
+          <t>V9</t>
+        </is>
+      </c>
+      <c r="B44" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:06</t>
+        </is>
+      </c>
+      <c r="C44" s="66" t="inlineStr">
+        <is>
+          <t>CTO face, bold text, logo bottom corner.</t>
+        </is>
+      </c>
+      <c r="D44" s="66" t="inlineStr">
+        <is>
+          <t>Cut your cloud bill. Free CTO session, 27 October.</t>
+        </is>
+      </c>
+      <c r="E44" s="66" t="inlineStr">
+        <is>
+          <t>Free CTO session · 27 Oct · Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="95" t="inlineStr">
+        <is>
+          <t>V10: Countdown, 10 s × 3 versions, 9:16 + 4:5</t>
+        </is>
+      </c>
+      <c r="B45" s="95" t="n"/>
+      <c r="C45" s="95" t="n"/>
+      <c r="D45" s="95" t="n"/>
+      <c r="E45" s="95" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="67" t="inlineStr">
+        <is>
+          <t>V10</t>
+        </is>
+      </c>
+      <c r="B46" s="66" t="inlineStr">
+        <is>
+          <t>0:00–0:03</t>
+        </is>
+      </c>
+      <c r="C46" s="66" t="inlineStr">
+        <is>
+          <t>Big number animation.</t>
+        </is>
+      </c>
+      <c r="D46" s="66" t="inlineStr">
+        <is>
+          <t>(music)</t>
+        </is>
+      </c>
+      <c r="E46" s="66" t="inlineStr">
+        <is>
+          <t>3 DAYS LEFT / TOMORROW / TODAY 4 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="67" t="inlineStr">
+        <is>
+          <t>V10</t>
+        </is>
+      </c>
+      <c r="B47" s="66" t="inlineStr">
+        <is>
+          <t>0:03–0:08</t>
+        </is>
+      </c>
+      <c r="C47" s="66" t="inlineStr">
+        <is>
+          <t>Speaker faces.</t>
+        </is>
+      </c>
+      <c r="D47" s="66" t="inlineStr">
+        <is>
+          <t>(music)</t>
+        </is>
+      </c>
+      <c r="E47" s="66" t="inlineStr">
+        <is>
+          <t>AI Is Eating Your Cloud Bill · Live bill teardown</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="67" t="inlineStr">
+        <is>
+          <t>V10</t>
+        </is>
+      </c>
+      <c r="B48" s="66" t="inlineStr">
+        <is>
+          <t>0:08–0:10</t>
+        </is>
+      </c>
+      <c r="C48" s="66" t="inlineStr">
+        <is>
+          <t>Button.</t>
+        </is>
+      </c>
+      <c r="D48" s="66" t="inlineStr">
+        <is>
+          <t>(music)</t>
+        </is>
+      </c>
+      <c r="E48" s="66" t="inlineStr">
+        <is>
+          <t>Register free →</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="74" t="inlineStr">
+        <is>
+          <t>Shoot checklist: lapel mic, window light or ring light, plain background with the Zarthi logo small, 3 outfits not needed (1 is fine), record each script 2–3 times, shoot vertical (9:16) and horizontal (16:9) versions of V3 and V4.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1894,7 +3527,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2033,10 +3666,10 @@
           <t>CTO + CEO</t>
         </is>
       </c>
-      <c r="J4" s="94" t="n">
+      <c r="J4" s="125" t="n">
         <v>46303</v>
       </c>
-      <c r="K4" s="94" t="n">
+      <c r="K4" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2086,10 +3719,10 @@
           <t>CTO</t>
         </is>
       </c>
-      <c r="J5" s="94" t="n">
+      <c r="J5" s="125" t="n">
         <v>46303</v>
       </c>
-      <c r="K5" s="94" t="n">
+      <c r="K5" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2139,10 +3772,10 @@
           <t>CTO</t>
         </is>
       </c>
-      <c r="J6" s="94" t="n">
+      <c r="J6" s="125" t="n">
         <v>46303</v>
       </c>
-      <c r="K6" s="94" t="n">
+      <c r="K6" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2192,10 +3825,10 @@
           <t>CEO</t>
         </is>
       </c>
-      <c r="J7" s="94" t="n">
+      <c r="J7" s="125" t="n">
         <v>46303</v>
       </c>
-      <c r="K7" s="94" t="n">
+      <c r="K7" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2245,10 +3878,10 @@
           <t>Editor</t>
         </is>
       </c>
-      <c r="J8" s="94" t="n">
+      <c r="J8" s="125" t="n">
         <v>46303</v>
       </c>
-      <c r="K8" s="94" t="n">
+      <c r="K8" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2298,10 +3931,10 @@
           <t>CTO</t>
         </is>
       </c>
-      <c r="J9" s="94" t="n">
+      <c r="J9" s="125" t="n">
         <v>46303</v>
       </c>
-      <c r="K9" s="94" t="n">
+      <c r="K9" s="125" t="n">
         <v>46309</v>
       </c>
     </row>
@@ -2351,10 +3984,10 @@
           <t>Zarthi engineer</t>
         </is>
       </c>
-      <c r="J10" s="94" t="n">
+      <c r="J10" s="125" t="n">
         <v>46308</v>
       </c>
-      <c r="K10" s="94" t="n">
+      <c r="K10" s="125" t="n">
         <v>46309</v>
       </c>
     </row>
@@ -2404,10 +4037,10 @@
           <t>CEO + CTO</t>
         </is>
       </c>
-      <c r="J11" s="94" t="n">
+      <c r="J11" s="125" t="n">
         <v>46308</v>
       </c>
-      <c r="K11" s="94" t="n">
+      <c r="K11" s="125" t="n">
         <v>46313</v>
       </c>
     </row>
@@ -2457,10 +4090,10 @@
           <t>Editor</t>
         </is>
       </c>
-      <c r="J12" s="94" t="n">
+      <c r="J12" s="125" t="n">
         <v>46313</v>
       </c>
-      <c r="K12" s="94" t="n">
+      <c r="K12" s="125" t="n">
         <v>46316</v>
       </c>
     </row>
@@ -2510,10 +4143,10 @@
           <t>Editor</t>
         </is>
       </c>
-      <c r="J13" s="94" t="n">
+      <c r="J13" s="125" t="n">
         <v>46317</v>
       </c>
-      <c r="K13" s="94" t="n">
+      <c r="K13" s="125" t="n">
         <v>46319</v>
       </c>
     </row>
@@ -2563,10 +4196,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J14" s="94" t="n">
+      <c r="J14" s="125" t="n">
         <v>46302</v>
       </c>
-      <c r="K14" s="94" t="n">
+      <c r="K14" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2616,10 +4249,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J15" s="94" t="n">
+      <c r="J15" s="125" t="n">
         <v>46302</v>
       </c>
-      <c r="K15" s="94" t="n">
+      <c r="K15" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2669,10 +4302,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J16" s="94" t="n">
+      <c r="J16" s="125" t="n">
         <v>46302</v>
       </c>
-      <c r="K16" s="94" t="n">
+      <c r="K16" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2722,10 +4355,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J17" s="94" t="n">
+      <c r="J17" s="125" t="n">
         <v>46307</v>
       </c>
-      <c r="K17" s="94" t="n">
+      <c r="K17" s="125" t="n">
         <v>46309</v>
       </c>
     </row>
@@ -2775,10 +4408,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J18" s="94" t="n">
+      <c r="J18" s="125" t="n">
         <v>46314</v>
       </c>
-      <c r="K18" s="94" t="n">
+      <c r="K18" s="125" t="n">
         <v>46315</v>
       </c>
     </row>
@@ -2828,10 +4461,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J19" s="94" t="n">
+      <c r="J19" s="125" t="n">
         <v>46312</v>
       </c>
-      <c r="K19" s="94" t="n">
+      <c r="K19" s="125" t="n">
         <v>46313</v>
       </c>
     </row>
@@ -2881,10 +4514,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J20" s="94" t="n">
+      <c r="J20" s="125" t="n">
         <v>46302</v>
       </c>
-      <c r="K20" s="94" t="n">
+      <c r="K20" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -2934,10 +4567,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J21" s="94" t="n">
+      <c r="J21" s="125" t="n">
         <v>46307</v>
       </c>
-      <c r="K21" s="94" t="n">
+      <c r="K21" s="125" t="n">
         <v>46309</v>
       </c>
     </row>
@@ -2987,10 +4620,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J22" s="94" t="n">
+      <c r="J22" s="125" t="n">
         <v>46311</v>
       </c>
-      <c r="K22" s="94" t="n">
+      <c r="K22" s="125" t="n">
         <v>46313</v>
       </c>
     </row>
@@ -3040,10 +4673,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J23" s="94" t="n">
+      <c r="J23" s="125" t="n">
         <v>46303</v>
       </c>
-      <c r="K23" s="94" t="n">
+      <c r="K23" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -3093,10 +4726,10 @@
           <t>Shourya</t>
         </is>
       </c>
-      <c r="J24" s="94" t="n">
+      <c r="J24" s="125" t="n">
         <v>46302</v>
       </c>
-      <c r="K24" s="94" t="n">
+      <c r="K24" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -3146,10 +4779,10 @@
           <t>Designer</t>
         </is>
       </c>
-      <c r="J25" s="94" t="n">
+      <c r="J25" s="125" t="n">
         <v>46303</v>
       </c>
-      <c r="K25" s="94" t="n">
+      <c r="K25" s="125" t="n">
         <v>46304</v>
       </c>
     </row>
@@ -3194,7 +4827,7 @@
     </row>
     <row r="30">
       <c r="A30" s="66" t="inlineStr"/>
-      <c r="B30" s="97" t="n">
+      <c r="B30" s="126" t="n">
         <v>46304</v>
       </c>
       <c r="C30" s="67" t="inlineStr">
@@ -3217,7 +4850,7 @@
     </row>
     <row r="31">
       <c r="A31" s="66" t="inlineStr"/>
-      <c r="B31" s="97" t="n">
+      <c r="B31" s="126" t="n">
         <v>46309</v>
       </c>
       <c r="C31" s="67" t="inlineStr">
@@ -3240,7 +4873,7 @@
     </row>
     <row r="32">
       <c r="A32" s="66" t="inlineStr"/>
-      <c r="B32" s="97" t="n">
+      <c r="B32" s="126" t="n">
         <v>46313</v>
       </c>
       <c r="C32" s="67" t="inlineStr">
@@ -3263,7 +4896,7 @@
     </row>
     <row r="33">
       <c r="A33" s="66" t="inlineStr"/>
-      <c r="B33" s="97" t="n">
+      <c r="B33" s="126" t="n">
         <v>46316</v>
       </c>
       <c r="C33" s="67" t="inlineStr">
@@ -3286,7 +4919,7 @@
     </row>
     <row r="34">
       <c r="A34" s="66" t="inlineStr"/>
-      <c r="B34" s="97" t="n">
+      <c r="B34" s="126" t="n">
         <v>46319</v>
       </c>
       <c r="C34" s="67" t="inlineStr">
@@ -3439,7 +5072,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3843,7 +5476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4590,7 +6223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4678,7 +6311,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="97" t="n">
+      <c r="A4" s="126" t="n">
         <v>46304</v>
       </c>
       <c r="B4" s="66" t="str">
@@ -4721,7 +6354,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="97" t="n">
+      <c r="A5" s="126" t="n">
         <v>46305</v>
       </c>
       <c r="B5" s="66" t="str">
@@ -4756,7 +6389,7 @@
       <c r="J5" s="66" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="97" t="n">
+      <c r="A6" s="126" t="n">
         <v>46306</v>
       </c>
       <c r="B6" s="66" t="str">
@@ -4791,7 +6424,7 @@
       <c r="J6" s="66" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="97" t="n">
+      <c r="A7" s="126" t="n">
         <v>46307</v>
       </c>
       <c r="B7" s="66" t="str">
@@ -4830,7 +6463,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="97" t="n">
+      <c r="A8" s="126" t="n">
         <v>46308</v>
       </c>
       <c r="B8" s="66" t="str">
@@ -4873,7 +6506,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="97" t="n">
+      <c r="A9" s="126" t="n">
         <v>46309</v>
       </c>
       <c r="B9" s="66" t="str">
@@ -4916,7 +6549,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="97" t="n">
+      <c r="A10" s="126" t="n">
         <v>46310</v>
       </c>
       <c r="B10" s="66" t="str">
@@ -4951,7 +6584,7 @@
       <c r="J10" s="66" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="97" t="n">
+      <c r="A11" s="126" t="n">
         <v>46311</v>
       </c>
       <c r="B11" s="66" t="str">
@@ -4986,7 +6619,7 @@
       <c r="J11" s="66" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="97" t="n">
+      <c r="A12" s="126" t="n">
         <v>46312</v>
       </c>
       <c r="B12" s="66" t="str">
@@ -5021,7 +6654,7 @@
       <c r="J12" s="66" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="97" t="n">
+      <c r="A13" s="126" t="n">
         <v>46313</v>
       </c>
       <c r="B13" s="66" t="str">
@@ -5060,7 +6693,7 @@
       <c r="J13" s="66" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="97" t="n">
+      <c r="A14" s="126" t="n">
         <v>46314</v>
       </c>
       <c r="B14" s="66" t="str">
@@ -5099,7 +6732,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="97" t="n">
+      <c r="A15" s="126" t="n">
         <v>46315</v>
       </c>
       <c r="B15" s="66" t="str">
@@ -5138,7 +6771,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="97" t="n">
+      <c r="A16" s="126" t="n">
         <v>46316</v>
       </c>
       <c r="B16" s="66" t="str">
@@ -5177,7 +6810,7 @@
       <c r="J16" s="66" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="97" t="n">
+      <c r="A17" s="126" t="n">
         <v>46317</v>
       </c>
       <c r="B17" s="66" t="str">
@@ -5216,7 +6849,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="97" t="n">
+      <c r="A18" s="126" t="n">
         <v>46318</v>
       </c>
       <c r="B18" s="66" t="str">
@@ -5255,7 +6888,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="97" t="n">
+      <c r="A19" s="126" t="n">
         <v>46319</v>
       </c>
       <c r="B19" s="66" t="str">
@@ -5298,7 +6931,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="97" t="n">
+      <c r="A20" s="126" t="n">
         <v>46320</v>
       </c>
       <c r="B20" s="66" t="str">
@@ -5333,7 +6966,7 @@
       <c r="J20" s="66" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="97" t="n">
+      <c r="A21" s="126" t="n">
         <v>46321</v>
       </c>
       <c r="B21" s="66" t="str">
@@ -5422,7 +7055,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF262626"/>
@@ -5821,7 +7454,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFB42A"/>
@@ -6226,7 +7859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF262626"/>
@@ -7571,6 +9204,373 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42.28515625" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" style="37" min="2" max="2"/>
+    <col width="59.85546875" customWidth="1" style="37" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="47" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B2" s="47" t="inlineStr">
+        <is>
+          <t>Promise statement</t>
+        </is>
+      </c>
+      <c r="C2" s="54" t="n"/>
+      <c r="D2" s="54" t="n"/>
+      <c r="E2" s="54" t="n"/>
+      <c r="F2" s="54" t="n"/>
+      <c r="G2" s="54" t="n"/>
+      <c r="H2" s="55" t="n"/>
+    </row>
+    <row r="3" ht="23.25" customHeight="1">
+      <c r="A3" s="56" t="inlineStr">
+        <is>
+          <t>AI Is Eating Your Cloud Bill: How SRE &amp; DevOps Teams Cut Kubernetes and AI Costs</t>
+        </is>
+      </c>
+      <c r="B3" s="56" t="inlineStr">
+        <is>
+          <t>In 45 minutes, see the 5 places cloud money leaks in Kubernetes and AI workloads, and the fixes your team can ship this sprint, with a live teardown of real (anonymised) cloud bills.</t>
+        </is>
+      </c>
+      <c r="C3" s="54" t="n"/>
+      <c r="D3" s="54" t="n"/>
+      <c r="E3" s="54" t="n"/>
+      <c r="F3" s="54" t="n"/>
+      <c r="G3" s="54" t="n"/>
+      <c r="H3" s="55" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="34" t="n"/>
+      <c r="B4" s="53" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="C4" s="53" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>Experience</t>
+        </is>
+      </c>
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t>3–15 years of total experience (pilot: wider net)</t>
+        </is>
+      </c>
+      <c r="C5" s="56" t="inlineStr">
+        <is>
+          <t>Freshers and students; job seekers</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30.75" customHeight="1">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>Seniority</t>
+        </is>
+      </c>
+      <c r="B6" s="56" t="inlineStr">
+        <is>
+          <t>SRE, DevOps, cloud, platform and backend engineers working on cloud, plus their leads and managers</t>
+        </is>
+      </c>
+      <c r="C6" s="56" t="inlineStr">
+        <is>
+          <t>C-suite (reached separately through direct outreach)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30.75" customHeight="1">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>Company type</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="inlineStr">
+        <is>
+          <t>Product and SaaS companies, GCCs, digital-first businesses (fintech, e-commerce, edtech, healthtech), in-house tech teams of enterprises (BFSI, healthcare, retail, manufacturing)</t>
+        </is>
+      </c>
+      <c r="C7" s="50" t="inlineStr">
+        <is>
+          <t>AWS partners and cloud MSPs (competitors). IT-services / outsourcing firms: CEO decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Company size</t>
+        </is>
+      </c>
+      <c r="B8" s="50" t="inlineStr">
+        <is>
+          <t>50+ employees (existing MQL gate)</t>
+        </is>
+      </c>
+      <c r="C8" s="50" t="inlineStr">
+        <is>
+          <t>Under 50 employees</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>Geography</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="inlineStr">
+        <is>
+          <t>India: Bengaluru, Hyderabad, Pune, Delhi-NCR, Chennai, Mumbai</t>
+        </is>
+      </c>
+      <c r="C9" s="50" t="inlineStr">
+        <is>
+          <t>Outside India for this first episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B10" s="50" t="inlineStr">
+        <is>
+          <t>Business email only</t>
+        </is>
+      </c>
+      <c r="C10" s="50" t="inlineStr">
+        <is>
+          <t>Gmail, Yahoo, Outlook and other personal domains</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B12" s="53" t="inlineStr">
+        <is>
+          <t>How</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="35" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="B13" s="56" t="inlineStr">
+        <is>
+          <t>Job titles + 3–15 years + company size 51+. Lead Gen Form + CTO Thought Leader Ads. 60 registrations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30.75" customHeight="1">
+      <c r="A14" s="35" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="B14" s="56" t="inlineStr">
+        <is>
+          <t>Age 24–45. Cloud/DevOps interests, developer interests, Advantage+ broad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="35" t="inlineStr">
+        <is>
+          <t>Own channels</t>
+        </is>
+      </c>
+      <c r="B15" s="56" t="inlineStr">
+        <is>
+          <t>Not used for acquisition. Email + WhatsApp only after registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="57" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="B16" s="58" t="inlineStr">
+        <is>
+          <t>Search (cost keywords) + Demand Gen (Discover, Gmail, YouTube feed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Funnel stage</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="59" t="inlineStr">
+        <is>
+          <t>Live attendees (target)</t>
+        </is>
+      </c>
+      <c r="B18" s="60">
+        <f>Funnel!B4</f>
+        <v>200.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="46" t="inlineStr">
+        <is>
+          <t>TNC Landing Page Best Practices: Video Clips, Speaker USPs, Tracking, and Retargeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="43" t="inlineStr">
+        <is>
+          <t>Form Question in lead form : Need to discuss this----comapny mail id, name number</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>date and time</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>for eg : 29 oct Sat 11:00 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B25" s="42" t="inlineStr">
+        <is>
+          <t>https://zoom.us/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="B26" s="58" t="inlineStr">
+        <is>
+          <t>Zoom Workplace Pro: INR 1,580 per user per month (host). For 200 live: Zoom Webinars 500, ₹11,610/month (Budget tab).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="40" t="inlineStr">
+        <is>
+          <t>Duration / Participants</t>
+        </is>
+      </c>
+      <c r="B27" s="61" t="inlineStr">
+        <is>
+          <t>Pro meetings hold 100; Webinars 500 holds 500 attendees</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>Local &amp; 10 GB cloud (per license)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>Mail</t>
+        </is>
+      </c>
+      <c r="B29" s="37" t="inlineStr">
+        <is>
+          <t>Zoom Mail and Calendar in the Zoom app</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30.75" customHeight="1">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>Clips</t>
+        </is>
+      </c>
+      <c r="B30" s="37" t="inlineStr">
+        <is>
+          <t>Effortlessly create, edit, and share short videos. Stored clips are easily discoverable, boosting engagement / Unlimited</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B2:H2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFB42A"/>
@@ -8732,7 +10732,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF262626"/>
@@ -9053,7 +11053,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF262626"/>
@@ -9556,7 +11556,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFB42A"/>
@@ -10263,10 +12263,10 @@
           <t>1. Test</t>
         </is>
       </c>
-      <c r="B27" s="89" t="n">
+      <c r="B27" s="123" t="n">
         <v>46304</v>
       </c>
-      <c r="C27" s="89" t="n">
+      <c r="C27" s="123" t="n">
         <v>46308</v>
       </c>
       <c r="D27" s="90">
@@ -10313,10 +12313,10 @@
           <t>2. Scale</t>
         </is>
       </c>
-      <c r="B28" s="89" t="n">
+      <c r="B28" s="123" t="n">
         <v>46309</v>
       </c>
-      <c r="C28" s="89" t="n">
+      <c r="C28" s="123" t="n">
         <v>46318</v>
       </c>
       <c r="D28" s="90">
@@ -10363,10 +12363,10 @@
           <t>3. Last call</t>
         </is>
       </c>
-      <c r="B29" s="89" t="n">
+      <c r="B29" s="123" t="n">
         <v>46319</v>
       </c>
-      <c r="C29" s="89" t="n">
+      <c r="C29" s="123" t="n">
         <v>46321</v>
       </c>
       <c r="D29" s="90">
@@ -10413,11 +12413,11 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B30" s="91">
+      <c r="B30" s="124">
         <f>B27</f>
         <v>46304.0</v>
       </c>
-      <c r="C30" s="91">
+      <c r="C30" s="124">
         <f>C29</f>
         <v>46321.0</v>
       </c>
@@ -10710,7 +12710,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10830,7 +12830,7 @@
           <t>CTO + designer</t>
         </is>
       </c>
-      <c r="I4" s="94" t="n">
+      <c r="I4" s="125" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -10873,7 +12873,7 @@
           <t>Shourya</t>
         </is>
       </c>
-      <c r="I5" s="94" t="n">
+      <c r="I5" s="125" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -10916,7 +12916,7 @@
           <t>CTO team</t>
         </is>
       </c>
-      <c r="I6" s="94" t="n">
+      <c r="I6" s="125" t="n">
         <v>46317</v>
       </c>
     </row>
@@ -10959,7 +12959,7 @@
           <t>Shourya</t>
         </is>
       </c>
-      <c r="I7" s="94" t="n">
+      <c r="I7" s="125" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -11002,7 +13002,7 @@
           <t>CTO</t>
         </is>
       </c>
-      <c r="I8" s="94" t="n">
+      <c r="I8" s="125" t="n">
         <v>46318</v>
       </c>
     </row>
@@ -11045,7 +13045,7 @@
           <t>Shourya</t>
         </is>
       </c>
-      <c r="I9" s="94" t="n">
+      <c r="I9" s="125" t="n">
         <v>46318</v>
       </c>
     </row>
@@ -11088,7 +13088,7 @@
           <t>Shourya</t>
         </is>
       </c>
-      <c r="I10" s="94" t="n">
+      <c r="I10" s="125" t="n">
         <v>46318</v>
       </c>
     </row>
@@ -11131,7 +13131,7 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="I11" s="94" t="n">
+      <c r="I11" s="125" t="n">
         <v>46318</v>
       </c>
     </row>
@@ -11174,7 +13174,7 @@
           <t>Shourya</t>
         </is>
       </c>
-      <c r="I12" s="94" t="n">
+      <c r="I12" s="125" t="n">
         <v>46321</v>
       </c>
     </row>
@@ -11217,7 +13217,7 @@
           <t>Shourya</t>
         </is>
       </c>
-      <c r="I13" s="94" t="n">
+      <c r="I13" s="125" t="n">
         <v>46303</v>
       </c>
     </row>
@@ -11287,7 +13287,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11426,11 +13426,11 @@
       <c r="G4" s="90" t="n">
         <v>4</v>
       </c>
-      <c r="H4" s="94">
+      <c r="H4" s="125">
         <f>Budget!B27</f>
         <v>46304.0</v>
       </c>
-      <c r="I4" s="94">
+      <c r="I4" s="125">
         <f>Budget!C29</f>
         <v>46321.0</v>
       </c>
@@ -11486,11 +13486,11 @@
       <c r="G5" s="90" t="n">
         <v>4</v>
       </c>
-      <c r="H5" s="94">
+      <c r="H5" s="125">
         <f>Budget!B27</f>
         <v>46304.0</v>
       </c>
-      <c r="I5" s="94">
+      <c r="I5" s="125">
         <f>Budget!C29</f>
         <v>46321.0</v>
       </c>
@@ -11546,11 +13546,11 @@
       <c r="G6" s="90" t="n">
         <v>3</v>
       </c>
-      <c r="H6" s="94">
+      <c r="H6" s="125">
         <f>Budget!B27</f>
         <v>46304.0</v>
       </c>
-      <c r="I6" s="94">
+      <c r="I6" s="125">
         <f>Budget!C29</f>
         <v>46321.0</v>
       </c>
@@ -11606,11 +13606,11 @@
       <c r="G7" s="90" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="94">
+      <c r="H7" s="125">
         <f>Budget!B28</f>
         <v>46309.0</v>
       </c>
-      <c r="I7" s="94">
+      <c r="I7" s="125">
         <f>Budget!C29</f>
         <v>46321.0</v>
       </c>
@@ -11666,11 +13666,11 @@
       <c r="G8" s="90" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="94">
+      <c r="H8" s="125">
         <f>Budget!B27</f>
         <v>46304.0</v>
       </c>
-      <c r="I8" s="94">
+      <c r="I8" s="125">
         <f>Budget!C29</f>
         <v>46321.0</v>
       </c>
@@ -11726,11 +13726,11 @@
       <c r="G9" s="90" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="94">
+      <c r="H9" s="125">
         <f>Budget!B27</f>
         <v>46304.0</v>
       </c>
-      <c r="I9" s="94">
+      <c r="I9" s="125">
         <f>Budget!C29</f>
         <v>46321.0</v>
       </c>
@@ -11786,11 +13786,11 @@
       <c r="G10" s="90" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="94">
+      <c r="H10" s="125">
         <f>Budget!B27</f>
         <v>46304.0</v>
       </c>
-      <c r="I10" s="94">
+      <c r="I10" s="125">
         <f>Budget!C29</f>
         <v>46321.0</v>
       </c>
@@ -11998,7 +13998,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13398,1129 +15398,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:E50"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="62" t="inlineStr">
-        <is>
-          <t>Video scripts: every video, scene by scene</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="74" t="inlineStr">
-        <is>
-          <t>One 2-hour shoot (Mon 5 or Tue 6 Oct) covers V1–V4, V6 and V8. Add burned-in captions to every video. [CTO name] = replace with the real name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="63" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="B3" s="63" t="inlineStr">
-        <is>
-          <t>Time</t>
-        </is>
-      </c>
-      <c r="C3" s="63" t="inlineStr">
-        <is>
-          <t>Shot / visual</t>
-        </is>
-      </c>
-      <c r="D3" s="63" t="inlineStr">
-        <is>
-          <t>Voiceover (exact words)</t>
-        </is>
-      </c>
-      <c r="E3" s="63" t="inlineStr">
-        <is>
-          <t>On-screen text</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="95" t="inlineStr">
-        <is>
-          <t>V1: Main VSL, 3–3.5 min, 16:9 (landing page)</t>
-        </is>
-      </c>
-      <c r="B4" s="95" t="n"/>
-      <c r="C4" s="95" t="n"/>
-      <c r="D4" s="95" t="n"/>
-      <c r="E4" s="95" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="67" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="B5" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:10</t>
-        </is>
-      </c>
-      <c r="C5" s="66" t="inlineStr">
-        <is>
-          <t>CTO close-up, office background. Cut-in: a monthly cost graph rising.</t>
-        </is>
-      </c>
-      <c r="D5" s="66" t="inlineStr">
-        <is>
-          <t>Your cloud bill went up again this month. Traffic didn't. Somewhere in your clusters, money is leaking, and in most teams nobody owns finding it.</t>
-        </is>
-      </c>
-      <c r="E5" s="66" t="inlineStr">
-        <is>
-          <t>Bill ↑. Traffic →. (example)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="67" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="B6" s="66" t="inlineStr">
-        <is>
-          <t>0:10–0:35</t>
-        </is>
-      </c>
-      <c r="C6" s="66" t="inlineStr">
-        <is>
-          <t>B-roll: Kubernetes dashboard, GPU usage graph, Slack message 'why is AWS so high?'</t>
-        </is>
-      </c>
-      <c r="D6" s="66" t="inlineStr">
-        <is>
-          <t>In 2026 it's getting worse. AI workloads, GPUs, idle dev clusters, oversized nodes. The State of FinOps report found 29% of cloud spend is wasted, and it went up for the first time in five years. And when finance asks why, they don't ask the vendor. They ask the SRE and DevOps team.</t>
-        </is>
-      </c>
-      <c r="E6" s="66" t="inlineStr">
-        <is>
-          <t>29% of cloud spend is wasted (State of FinOps 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="67" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="B7" s="66" t="inlineStr">
-        <is>
-          <t>0:35–1:05</t>
-        </is>
-      </c>
-      <c r="C7" s="66" t="inlineStr">
-        <is>
-          <t>CTO introduces himself; quick cut to CEO.</t>
-        </is>
-      </c>
-      <c r="D7" s="66" t="inlineStr">
-        <is>
-          <t>I'm [CTO name], CTO at Zarthi. I've spent 15 years building cloud platforms, including at Microsoft. My team reviews cloud setups for Indian product companies every week, and the same five leaks show up almost every time. CEO: That's why we started Think Like a CTO: free sessions for engineers who want to make the calls, not just close the tickets.</t>
-        </is>
-      </c>
-      <c r="E7" s="66" t="inlineStr">
-        <is>
-          <t>[CTO name] · CTO, Zarthi · ex-Microsoft</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="67" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="B8" s="66" t="inlineStr">
-        <is>
-          <t>1:05–1:50</t>
-        </is>
-      </c>
-      <c r="C8" s="66" t="inlineStr">
-        <is>
-          <t>Screen recording: 'kubectl top pods' next to the requests in a deployment YAML; requests highlighted in red.</t>
-        </is>
-      </c>
-      <c r="D8" s="66" t="inlineStr">
-        <is>
-          <t>Let me give you leak number one right now. Idle and oversized compute. Pull the CPU and memory requests for your top ten workloads and compare them with what they actually use. If requests are double the usage, you're paying for air. Fix it with rightsizing and autoscaling. That's one of five.</t>
-        </is>
-      </c>
-      <c r="E8" s="66" t="inlineStr">
-        <is>
-          <t>Leak #1: requests ≫ usage = paying for air</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="67" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="B9" s="66" t="inlineStr">
-        <is>
-          <t>1:50–2:30</t>
-        </is>
-      </c>
-      <c r="C9" s="66" t="inlineStr">
-        <is>
-          <t>CTO on camera; graphics pop in for each benefit.</t>
-        </is>
-      </c>
-      <c r="D9" s="66" t="inlineStr">
-        <is>
-          <t>On Tuesday, 27 October at 4 PM, I'll walk through all five leaks, including GPU and AI inference costs, and tear down real, anonymised cloud bills that you send in. You get the 27-point Cost Leak Checklist the moment you register. Join live and you also get the full playbook, a certificate, and a chance to win vouchers. The first 300 people also get our AI Cost Guardrails Pack.</t>
-        </is>
-      </c>
-      <c r="E9" s="66" t="inlineStr">
-        <is>
-          <t>Free checklist now · Playbook + certificate + lucky draw live</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="67" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="B10" s="66" t="inlineStr">
-        <is>
-          <t>2:30–2:55</t>
-        </is>
-      </c>
-      <c r="C10" s="66" t="inlineStr">
-        <is>
-          <t>CTO, two-column 'For / Not for' graphic.</t>
-        </is>
-      </c>
-      <c r="D10" s="66" t="inlineStr">
-        <is>
-          <t>This is for SREs, DevOps, platform and cloud engineers, and developers who run things on AWS, Azure or GCP. It's not a beginner course, and it's not a sales pitch. There's no product demo.</t>
-        </is>
-      </c>
-      <c r="E10" s="66" t="inlineStr">
-        <is>
-          <t>For: SRE · DevOps · Platform · Cloud · Developers</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="67" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="B11" s="66" t="inlineStr">
-        <is>
-          <t>2:55–3:20</t>
-        </is>
-      </c>
-      <c r="C11" s="66" t="inlineStr">
-        <is>
-          <t>CTO points down; date card; form appears below the video.</t>
-        </is>
-      </c>
-      <c r="D11" s="66" t="inlineStr">
-        <is>
-          <t>Forty-five minutes. Free. Register below, and add your cloud bill question in the form. If yours is picked, we tear it down live. See you on the 27th.</t>
-        </is>
-      </c>
-      <c r="E11" s="66" t="inlineStr">
-        <is>
-          <t>Tue 27 Oct · 4 PM IST · Free · Register below ↓</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="95" t="inlineStr">
-        <is>
-          <t>V2: 60-second cut, 16:9 / 1:1 / 9:16 (Google Demand Gen, LinkedIn, Meta)</t>
-        </is>
-      </c>
-      <c r="B12" s="95" t="n"/>
-      <c r="C12" s="95" t="n"/>
-      <c r="D12" s="95" t="n"/>
-      <c r="E12" s="95" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="67" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="B13" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:05</t>
-        </is>
-      </c>
-      <c r="C13" s="66" t="inlineStr">
-        <is>
-          <t>CTO close-up, bold caption.</t>
-        </is>
-      </c>
-      <c r="D13" s="66" t="inlineStr">
-        <is>
-          <t>29% of cloud spend is wasted. Here's where it hides in Kubernetes.</t>
-        </is>
-      </c>
-      <c r="E13" s="66" t="inlineStr">
-        <is>
-          <t>29% wasted</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="67" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="B14" s="66" t="inlineStr">
-        <is>
-          <t>0:05–0:20</t>
-        </is>
-      </c>
-      <c r="C14" s="66" t="inlineStr">
-        <is>
-          <t>B-roll of dashboards; CTO voice.</t>
-        </is>
-      </c>
-      <c r="D14" s="66" t="inlineStr">
-        <is>
-          <t>Idle dev clusters. Pods asking for twice the CPU they use. GPUs sitting at 10%. And the bill lands on the SRE and DevOps team.</t>
-        </is>
-      </c>
-      <c r="E14" s="66" t="inlineStr">
-        <is>
-          <t>Idle clusters · Oversized pods · Idle GPUs</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="67" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="B15" s="66" t="inlineStr">
-        <is>
-          <t>0:20–0:40</t>
-        </is>
-      </c>
-      <c r="C15" s="66" t="inlineStr">
-        <is>
-          <t>Screen: kubectl top vs YAML requests.</t>
-        </is>
-      </c>
-      <c r="D15" s="66" t="inlineStr">
-        <is>
-          <t>Quick check: compare requests with real usage for your top ten workloads. Double? You're paying for air.</t>
-        </is>
-      </c>
-      <c r="E15" s="66" t="inlineStr">
-        <is>
-          <t>Requests vs usage: check yours</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="67" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="B16" s="66" t="inlineStr">
-        <is>
-          <t>0:40–0:55</t>
-        </is>
-      </c>
-      <c r="C16" s="66" t="inlineStr">
-        <is>
-          <t>CTO; benefit graphics.</t>
-        </is>
-      </c>
-      <c r="D16" s="66" t="inlineStr">
-        <is>
-          <t>On 27 October I'll show all five leaks and tear down real bills live. Register and get our 27-point Cost Leak Checklist free.</t>
-        </is>
-      </c>
-      <c r="E16" s="66" t="inlineStr">
-        <is>
-          <t>Free checklist on sign-up</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="67" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="B17" s="66" t="inlineStr">
-        <is>
-          <t>0:55–1:00</t>
-        </is>
-      </c>
-      <c r="C17" s="66" t="inlineStr">
-        <is>
-          <t>End card with date and button.</t>
-        </is>
-      </c>
-      <c r="D17" s="66" t="inlineStr">
-        <is>
-          <t>Free, 45 minutes. Link below.</t>
-        </is>
-      </c>
-      <c r="E17" s="66" t="inlineStr">
-        <is>
-          <t>Tue 27 Oct · 4 PM · Register</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="95" t="inlineStr">
-        <is>
-          <t>V3: CTO talking head, 30 s, 9:16 + 4:5 (Meta, LinkedIn)</t>
-        </is>
-      </c>
-      <c r="B18" s="95" t="n"/>
-      <c r="C18" s="95" t="n"/>
-      <c r="D18" s="95" t="n"/>
-      <c r="E18" s="95" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="67" t="inlineStr">
-        <is>
-          <t>V3</t>
-        </is>
-      </c>
-      <c r="B19" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:03</t>
-        </is>
-      </c>
-      <c r="C19" s="66" t="inlineStr">
-        <is>
-          <t>CTO, phone camera, eye level.</t>
-        </is>
-      </c>
-      <c r="D19" s="66" t="inlineStr">
-        <is>
-          <t>Three places your Kubernetes bill leaks. Number two surprises everyone.</t>
-        </is>
-      </c>
-      <c r="E19" s="66" t="inlineStr">
-        <is>
-          <t>3 Kubernetes bill leaks</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="67" t="inlineStr">
-        <is>
-          <t>V3</t>
-        </is>
-      </c>
-      <c r="B20" s="66" t="inlineStr">
-        <is>
-          <t>0:03–0:12</t>
-        </is>
-      </c>
-      <c r="C20" s="66" t="inlineStr">
-        <is>
-          <t>CTO counts on fingers.</t>
-        </is>
-      </c>
-      <c r="D20" s="66" t="inlineStr">
-        <is>
-          <t>One: pods asking for far more CPU than they use. Two: logs. Teams spend more storing debug logs than running the app.</t>
-        </is>
-      </c>
-      <c r="E20" s="66" t="inlineStr">
-        <is>
-          <t>1. Oversized pods  2. Log storage</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="67" t="inlineStr">
-        <is>
-          <t>V3</t>
-        </is>
-      </c>
-      <c r="B21" s="66" t="inlineStr">
-        <is>
-          <t>0:12–0:22</t>
-        </is>
-      </c>
-      <c r="C21" s="66" t="inlineStr">
-        <is>
-          <t>CTO.</t>
-        </is>
-      </c>
-      <c r="D21" s="66" t="inlineStr">
-        <is>
-          <t>Three: dev and staging clusters running all night and every weekend.</t>
-        </is>
-      </c>
-      <c r="E21" s="66" t="inlineStr">
-        <is>
-          <t>3. Clusters that never sleep</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="67" t="inlineStr">
-        <is>
-          <t>V3</t>
-        </is>
-      </c>
-      <c r="B22" s="66" t="inlineStr">
-        <is>
-          <t>0:22–0:30</t>
-        </is>
-      </c>
-      <c r="C22" s="66" t="inlineStr">
-        <is>
-          <t>CTO points to caption.</t>
-        </is>
-      </c>
-      <c r="D22" s="66" t="inlineStr">
-        <is>
-          <t>I'll show the other two, and the fixes, live on the 27th. Free. Link below.</t>
-        </is>
-      </c>
-      <c r="E22" s="66" t="inlineStr">
-        <is>
-          <t>Free live session · 27 Oct · 4 PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="95" t="inlineStr">
-        <is>
-          <t>V4: CEO talking head, 30 s, 4:5 + 1:1 (Meta, LinkedIn)</t>
-        </is>
-      </c>
-      <c r="B23" s="95" t="n"/>
-      <c r="C23" s="95" t="n"/>
-      <c r="D23" s="95" t="n"/>
-      <c r="E23" s="95" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="67" t="inlineStr">
-        <is>
-          <t>V4</t>
-        </is>
-      </c>
-      <c r="B24" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:04</t>
-        </is>
-      </c>
-      <c r="C24" s="66" t="inlineStr">
-        <is>
-          <t>CEO, office.</t>
-        </is>
-      </c>
-      <c r="D24" s="66" t="inlineStr">
-        <is>
-          <t>The engineers who get promoted fastest can explain the cloud bill.</t>
-        </is>
-      </c>
-      <c r="E24" s="66" t="inlineStr">
-        <is>
-          <t>Can you explain your cloud bill?</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="67" t="inlineStr">
-        <is>
-          <t>V4</t>
-        </is>
-      </c>
-      <c r="B25" s="66" t="inlineStr">
-        <is>
-          <t>0:04–0:18</t>
-        </is>
-      </c>
-      <c r="C25" s="66" t="inlineStr">
-        <is>
-          <t>CEO.</t>
-        </is>
-      </c>
-      <c r="D25" s="66" t="inlineStr">
-        <is>
-          <t>Not because they're accountants. Because when the bill jumps, the CTO needs someone who knows which service, which team, and which fix. That person gets trusted with bigger decisions.</t>
-        </is>
-      </c>
-      <c r="E25" s="66" t="inlineStr">
-        <is>
-          <t>Cost = a leadership skill</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="67" t="inlineStr">
-        <is>
-          <t>V4</t>
-        </is>
-      </c>
-      <c r="B26" s="66" t="inlineStr">
-        <is>
-          <t>0:18–0:30</t>
-        </is>
-      </c>
-      <c r="C26" s="66" t="inlineStr">
-        <is>
-          <t>CEO; date card.</t>
-        </is>
-      </c>
-      <c r="D26" s="66" t="inlineStr">
-        <is>
-          <t>Our CTO is teaching exactly that, free, on 27 October. SREs, DevOps and cloud engineers: register below.</t>
-        </is>
-      </c>
-      <c r="E26" s="66" t="inlineStr">
-        <is>
-          <t>Free · 27 Oct · 4 PM IST</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="95" t="inlineStr">
-        <is>
-          <t>V5: Myth vs fact reel, 15 s, 9:16 (Meta Reels/Stories)</t>
-        </is>
-      </c>
-      <c r="B27" s="95" t="n"/>
-      <c r="C27" s="95" t="n"/>
-      <c r="D27" s="95" t="n"/>
-      <c r="E27" s="95" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="67" t="inlineStr">
-        <is>
-          <t>V5</t>
-        </is>
-      </c>
-      <c r="B28" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:04</t>
-        </is>
-      </c>
-      <c r="C28" s="66" t="inlineStr">
-        <is>
-          <t>Big text on a dark background, beat-synced.</t>
-        </is>
-      </c>
-      <c r="D28" s="66" t="inlineStr">
-        <is>
-          <t>(music only)</t>
-        </is>
-      </c>
-      <c r="E28" s="66" t="inlineStr">
-        <is>
-          <t>MYTH: Autoscaling saves money.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="67" t="inlineStr">
-        <is>
-          <t>V5</t>
-        </is>
-      </c>
-      <c r="B29" s="66" t="inlineStr">
-        <is>
-          <t>0:04–0:09</t>
-        </is>
-      </c>
-      <c r="C29" s="66" t="inlineStr">
-        <is>
-          <t>Text card + screenshot of a node pool.</t>
-        </is>
-      </c>
-      <c r="D29" s="66" t="inlineStr">
-        <is>
-          <t>(music only)</t>
-        </is>
-      </c>
-      <c r="E29" s="66" t="inlineStr">
-        <is>
-          <t>FACT: Autoscaling on oversized requests scales the waste too.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="67" t="inlineStr">
-        <is>
-          <t>V5</t>
-        </is>
-      </c>
-      <c r="B30" s="66" t="inlineStr">
-        <is>
-          <t>0:09–0:15</t>
-        </is>
-      </c>
-      <c r="C30" s="66" t="inlineStr">
-        <is>
-          <t>Speaker faces + date.</t>
-        </is>
-      </c>
-      <c r="D30" s="66" t="inlineStr">
-        <is>
-          <t>(music only)</t>
-        </is>
-      </c>
-      <c r="E30" s="66" t="inlineStr">
-        <is>
-          <t>5 leaks + live bill teardown · Free · 27 Oct · Register</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="95" t="inlineStr">
-        <is>
-          <t>V6: Whiteboard explainer, 45 s, 9:16 + 16:9</t>
-        </is>
-      </c>
-      <c r="B31" s="95" t="n"/>
-      <c r="C31" s="95" t="n"/>
-      <c r="D31" s="95" t="n"/>
-      <c r="E31" s="95" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="67" t="inlineStr">
-        <is>
-          <t>V6</t>
-        </is>
-      </c>
-      <c r="B32" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:05</t>
-        </is>
-      </c>
-      <c r="C32" s="66" t="inlineStr">
-        <is>
-          <t>CTO at a whiteboard, writes ₹100.</t>
-        </is>
-      </c>
-      <c r="D32" s="66" t="inlineStr">
-        <is>
-          <t>Follow 100 rupees of cloud spend and watch 29 disappear.</t>
-        </is>
-      </c>
-      <c r="E32" s="66" t="inlineStr">
-        <is>
-          <t>Where does ₹100 go?</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="67" t="inlineStr">
-        <is>
-          <t>V6</t>
-        </is>
-      </c>
-      <c r="B33" s="66" t="inlineStr">
-        <is>
-          <t>0:05–0:30</t>
-        </is>
-      </c>
-      <c r="C33" s="66" t="inlineStr">
-        <is>
-          <t>CTO draws boxes: compute, storage, data transfer, AI/GPU; crosses out parts.</t>
-        </is>
-      </c>
-      <c r="D33" s="66" t="inlineStr">
-        <is>
-          <t>Compute you reserved but don't use. Storage nobody deleted. Data moving between zones for no reason. GPUs waiting for jobs. Add it up: about 29 rupees of every 100.</t>
-        </is>
-      </c>
-      <c r="E33" s="66" t="inlineStr">
-        <is>
-          <t>Unused compute · Old storage · Cross-zone traffic · Idle GPUs</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="67" t="inlineStr">
-        <is>
-          <t>V6</t>
-        </is>
-      </c>
-      <c r="B34" s="66" t="inlineStr">
-        <is>
-          <t>0:30–0:45</t>
-        </is>
-      </c>
-      <c r="C34" s="66" t="inlineStr">
-        <is>
-          <t>CTO caps the marker.</t>
-        </is>
-      </c>
-      <c r="D34" s="66" t="inlineStr">
-        <is>
-          <t>On 27 October I'll show how to find each one in your own account, and fix it. Free. Register below.</t>
-        </is>
-      </c>
-      <c r="E34" s="66" t="inlineStr">
-        <is>
-          <t>Free · 27 Oct · 4 PM IST</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="95" t="inlineStr">
-        <is>
-          <t>V7: Engineer POV, 25 s, 9:16 (Meta Reels). Use only if the story is true; change the numbers to the real ones.</t>
-        </is>
-      </c>
-      <c r="B35" s="95" t="n"/>
-      <c r="C35" s="95" t="n"/>
-      <c r="D35" s="95" t="n"/>
-      <c r="E35" s="95" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="67" t="inlineStr">
-        <is>
-          <t>V7</t>
-        </is>
-      </c>
-      <c r="B36" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:04</t>
-        </is>
-      </c>
-      <c r="C36" s="66" t="inlineStr">
-        <is>
-          <t>Zarthi engineer, selfie, natural light.</t>
-        </is>
-      </c>
-      <c r="D36" s="66" t="inlineStr">
-        <is>
-          <t>Our staging clusters ran all night. Nobody used them after 8 PM.</t>
-        </is>
-      </c>
-      <c r="E36" s="66" t="inlineStr">
-        <is>
-          <t>Staging, running 24/7</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="67" t="inlineStr">
-        <is>
-          <t>V7</t>
-        </is>
-      </c>
-      <c r="B37" s="66" t="inlineStr">
-        <is>
-          <t>0:04–0:16</t>
-        </is>
-      </c>
-      <c r="C37" s="66" t="inlineStr">
-        <is>
-          <t>Engineer; screen of a cron schedule.</t>
-        </is>
-      </c>
-      <c r="D37" s="66" t="inlineStr">
-        <is>
-          <t>One scheduled scale-down at night and on weekends. Our staging bill dropped by about a third the next month.</t>
-        </is>
-      </c>
-      <c r="E37" s="66" t="inlineStr">
-        <is>
-          <t>1 schedule → staging bill ↓ (use real number)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="67" t="inlineStr">
-        <is>
-          <t>V7</t>
-        </is>
-      </c>
-      <c r="B38" s="66" t="inlineStr">
-        <is>
-          <t>0:16–0:25</t>
-        </is>
-      </c>
-      <c r="C38" s="66" t="inlineStr">
-        <is>
-          <t>Engineer.</t>
-        </is>
-      </c>
-      <c r="D38" s="66" t="inlineStr">
-        <is>
-          <t>Our CTO is sharing five fixes like this live on the 27th. It's free. Link below.</t>
-        </is>
-      </c>
-      <c r="E38" s="66" t="inlineStr">
-        <is>
-          <t>Free live session · 27 Oct</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="95" t="inlineStr">
-        <is>
-          <t>V8: CEO + CTO podcast clip, 40 s, 1:1 + 9:16</t>
-        </is>
-      </c>
-      <c r="B39" s="95" t="n"/>
-      <c r="C39" s="95" t="n"/>
-      <c r="D39" s="95" t="n"/>
-      <c r="E39" s="95" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="67" t="inlineStr">
-        <is>
-          <t>V8</t>
-        </is>
-      </c>
-      <c r="B40" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:05</t>
-        </is>
-      </c>
-      <c r="C40" s="66" t="inlineStr">
-        <is>
-          <t>Two-shot, mics visible.</t>
-        </is>
-      </c>
-      <c r="D40" s="66" t="inlineStr">
-        <is>
-          <t>CEO: Who owns the cloud bill in most teams?</t>
-        </is>
-      </c>
-      <c r="E40" s="66" t="inlineStr">
-        <is>
-          <t>Who owns the cloud bill?</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="67" t="inlineStr">
-        <is>
-          <t>V8</t>
-        </is>
-      </c>
-      <c r="B41" s="66" t="inlineStr">
-        <is>
-          <t>0:05–0:25</t>
-        </is>
-      </c>
-      <c r="C41" s="66" t="inlineStr">
-        <is>
-          <t>Close-up CTO.</t>
-        </is>
-      </c>
-      <c r="D41" s="66" t="inlineStr">
-        <is>
-          <t>CTO: Honestly? Nobody, until it doubles. Then it's suddenly the DevOps team's problem. The fix isn't a tool. It's making cost visible per team, with guardrails so nobody can launch a 64-core pod by accident.</t>
-        </is>
-      </c>
-      <c r="E41" s="66" t="inlineStr">
-        <is>
-          <t>Make cost visible · Add guardrails</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="67" t="inlineStr">
-        <is>
-          <t>V8</t>
-        </is>
-      </c>
-      <c r="B42" s="66" t="inlineStr">
-        <is>
-          <t>0:25–0:40</t>
-        </is>
-      </c>
-      <c r="C42" s="66" t="inlineStr">
-        <is>
-          <t>Two-shot, date card.</t>
-        </is>
-      </c>
-      <c r="D42" s="66" t="inlineStr">
-        <is>
-          <t>CEO: We're going deep on this live on the 27th. CTO: Bring your bill. We'll tear it down.</t>
-        </is>
-      </c>
-      <c r="E42" s="66" t="inlineStr">
-        <is>
-          <t>Free · 27 Oct · 4 PM IST</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="95" t="inlineStr">
-        <is>
-          <t>V9: Bumper, 6 s, 16:9 (Google Demand Gen video)</t>
-        </is>
-      </c>
-      <c r="B43" s="95" t="n"/>
-      <c r="C43" s="95" t="n"/>
-      <c r="D43" s="95" t="n"/>
-      <c r="E43" s="95" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="67" t="inlineStr">
-        <is>
-          <t>V9</t>
-        </is>
-      </c>
-      <c r="B44" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:06</t>
-        </is>
-      </c>
-      <c r="C44" s="66" t="inlineStr">
-        <is>
-          <t>CTO face, bold text, logo bottom corner.</t>
-        </is>
-      </c>
-      <c r="D44" s="66" t="inlineStr">
-        <is>
-          <t>Cut your cloud bill. Free CTO session, 27 October.</t>
-        </is>
-      </c>
-      <c r="E44" s="66" t="inlineStr">
-        <is>
-          <t>Free CTO session · 27 Oct · Register</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="95" t="inlineStr">
-        <is>
-          <t>V10: Countdown, 10 s × 3 versions, 9:16 + 4:5</t>
-        </is>
-      </c>
-      <c r="B45" s="95" t="n"/>
-      <c r="C45" s="95" t="n"/>
-      <c r="D45" s="95" t="n"/>
-      <c r="E45" s="95" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="67" t="inlineStr">
-        <is>
-          <t>V10</t>
-        </is>
-      </c>
-      <c r="B46" s="66" t="inlineStr">
-        <is>
-          <t>0:00–0:03</t>
-        </is>
-      </c>
-      <c r="C46" s="66" t="inlineStr">
-        <is>
-          <t>Big number animation.</t>
-        </is>
-      </c>
-      <c r="D46" s="66" t="inlineStr">
-        <is>
-          <t>(music)</t>
-        </is>
-      </c>
-      <c r="E46" s="66" t="inlineStr">
-        <is>
-          <t>3 DAYS LEFT / TOMORROW / TODAY 4 PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="67" t="inlineStr">
-        <is>
-          <t>V10</t>
-        </is>
-      </c>
-      <c r="B47" s="66" t="inlineStr">
-        <is>
-          <t>0:03–0:08</t>
-        </is>
-      </c>
-      <c r="C47" s="66" t="inlineStr">
-        <is>
-          <t>Speaker faces.</t>
-        </is>
-      </c>
-      <c r="D47" s="66" t="inlineStr">
-        <is>
-          <t>(music)</t>
-        </is>
-      </c>
-      <c r="E47" s="66" t="inlineStr">
-        <is>
-          <t>AI Is Eating Your Cloud Bill · Live bill teardown</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="67" t="inlineStr">
-        <is>
-          <t>V10</t>
-        </is>
-      </c>
-      <c r="B48" s="66" t="inlineStr">
-        <is>
-          <t>0:08–0:10</t>
-        </is>
-      </c>
-      <c r="C48" s="66" t="inlineStr">
-        <is>
-          <t>Button.</t>
-        </is>
-      </c>
-      <c r="D48" s="66" t="inlineStr">
-        <is>
-          <t>(music)</t>
-        </is>
-      </c>
-      <c r="E48" s="66" t="inlineStr">
-        <is>
-          <t>Register free →</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="74" t="inlineStr">
-        <is>
-          <t>Shoot checklist: lapel mic, window light or ring light, plain background with the Zarthi logo small, 3 outfits not needed (1 is fine), record each script 2–3 times, shoot vertical (9:16) and horizontal (16:9) versions of V3 and V4.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Audience Universe tab: reach by platform and Google Search capacity
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GGpsSZB9EZkEvXCwx9WBeN
</commit_message>
<xml_diff>
--- a/Zarthi_Webinar_CEO_Plan_22Sep26.xlsx
+++ b/Zarthi_Webinar_CEO_Plan_22Sep26.xlsx
@@ -10,24 +10,25 @@
     <sheet name="Overview" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Topics" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Audience" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Funnel" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Budget" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Offers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Ads Plan" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Ad Copy" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Video Scripts" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Image Ideas" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Creatives" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="VSL Funnel" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Email &amp; WhatsApp" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Daily Plan" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Timeline" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Decisions" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Checklist" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Audience Universe" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Funnel" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Budget" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Offers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Ads Plan" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Ad Copy" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Video Scripts" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Image Ideas" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Creatives" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="VSL Funnel" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Email &amp; WhatsApp" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Daily Plan" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Timeline" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Decisions" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Checklist" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Manager Summary'!$A$1:$E$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Checklist'!$A$3:$D$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Checklist'!$A$3:$D$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -201,7 +202,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -248,6 +249,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -391,7 +402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -713,6 +724,17 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="20" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1858,6 +1880,1408 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:G61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="62" t="inlineStr">
+        <is>
+          <t>Ad copy: Meta, LinkedIn and Google</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="74" t="inlineStr">
+        <is>
+          <t>Character counts are formulas so you can edit and check. Limits: Google headline 30, description 90; Demand Gen headline 40; LinkedIn headline 70.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="69" t="inlineStr">
+        <is>
+          <t>Meta (Facebook + Instagram)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="63" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B5" s="63" t="inlineStr">
+        <is>
+          <t>Angle</t>
+        </is>
+      </c>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t>Primary text</t>
+        </is>
+      </c>
+      <c r="D5" s="63" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="E5" s="63" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F5" s="63" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="G5" s="63" t="inlineStr">
+        <is>
+          <t>Use with</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>M-A</t>
+        </is>
+      </c>
+      <c r="B6" s="67" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="C6" s="66" t="inlineStr">
+        <is>
+          <t>29% of cloud spend is wasted, and it's rising again (State of FinOps 2026). On 27 Oct our CTO shows the 5 places it leaks in Kubernetes and AI workloads, with a live bill teardown. Free checklist when you register.</t>
+        </is>
+      </c>
+      <c r="D6" s="66" t="inlineStr">
+        <is>
+          <t>Find the 29% your cloud bill wastes</t>
+        </is>
+      </c>
+      <c r="E6" s="66" t="inlineStr">
+        <is>
+          <t>Free live session · 27 Oct · 4 PM IST</t>
+        </is>
+      </c>
+      <c r="F6" s="66" t="inlineStr">
+        <is>
+          <t>Sign up</t>
+        </is>
+      </c>
+      <c r="G6" s="66" t="inlineStr">
+        <is>
+          <t>V2, S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>M-B</t>
+        </is>
+      </c>
+      <c r="B7" s="67" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="C7" s="66" t="inlineStr">
+        <is>
+          <t>Bill up. Traffic flat. And somehow it's the DevOps team's problem. Learn how SREs find idle clusters, oversized pods and idle GPUs, and fix them this sprint.</t>
+        </is>
+      </c>
+      <c r="D7" s="66" t="inlineStr">
+        <is>
+          <t>Your cloud bill went up again?</t>
+        </is>
+      </c>
+      <c r="E7" s="66" t="inlineStr">
+        <is>
+          <t>45 min · Free · No sales pitch</t>
+        </is>
+      </c>
+      <c r="F7" s="66" t="inlineStr">
+        <is>
+          <t>Sign up</t>
+        </is>
+      </c>
+      <c r="G7" s="66" t="inlineStr">
+        <is>
+          <t>V3, S1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="67" t="inlineStr">
+        <is>
+          <t>M-C</t>
+        </is>
+      </c>
+      <c r="B8" s="67" t="inlineStr">
+        <is>
+          <t>Curiosity</t>
+        </is>
+      </c>
+      <c r="C8" s="66" t="inlineStr">
+        <is>
+          <t>3 places your Kubernetes bill leaks. Number 2 surprises almost everyone. Our CTO (ex-Microsoft, 15 yrs) covers all 5 live on 27 Oct.</t>
+        </is>
+      </c>
+      <c r="D8" s="66" t="inlineStr">
+        <is>
+          <t>3 Kubernetes bill leaks (no. 2!)</t>
+        </is>
+      </c>
+      <c r="E8" s="66" t="inlineStr">
+        <is>
+          <t>Free CTO session for engineers</t>
+        </is>
+      </c>
+      <c r="F8" s="66" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="G8" s="66" t="inlineStr">
+        <is>
+          <t>V3, C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="67" t="inlineStr">
+        <is>
+          <t>M-D</t>
+        </is>
+      </c>
+      <c r="B9" s="67" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="C9" s="66" t="inlineStr">
+        <is>
+          <t>Register free and get our 27-point Cloud &amp; Kubernetes Cost Leak Checklist right away. Join live on 27 Oct for the full playbook, a certificate and a ₹5,000 lucky draw.</t>
+        </is>
+      </c>
+      <c r="D9" s="66" t="inlineStr">
+        <is>
+          <t>Free 27-point Cost Leak Checklist</t>
+        </is>
+      </c>
+      <c r="E9" s="66" t="inlineStr">
+        <is>
+          <t>Instant download when you register</t>
+        </is>
+      </c>
+      <c r="F9" s="66" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="G9" s="66" t="inlineStr">
+        <is>
+          <t>S4, V1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="67" t="inlineStr">
+        <is>
+          <t>M-E</t>
+        </is>
+      </c>
+      <c r="B10" s="67" t="inlineStr">
+        <is>
+          <t>Career</t>
+        </is>
+      </c>
+      <c r="C10" s="66" t="inlineStr">
+        <is>
+          <t>The engineers who get promoted fastest can explain the cloud bill. Learn how a CTO reads one, live on 27 Oct. For SRE, DevOps, cloud and platform engineers.</t>
+        </is>
+      </c>
+      <c r="D10" s="66" t="inlineStr">
+        <is>
+          <t>Explain the bill. Get the promotion.</t>
+        </is>
+      </c>
+      <c r="E10" s="66" t="inlineStr">
+        <is>
+          <t>Think Like a CTO · Episode 1</t>
+        </is>
+      </c>
+      <c r="F10" s="66" t="inlineStr">
+        <is>
+          <t>Sign up</t>
+        </is>
+      </c>
+      <c r="G10" s="66" t="inlineStr">
+        <is>
+          <t>V4, C3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="67" t="inlineStr">
+        <is>
+          <t>M-F</t>
+        </is>
+      </c>
+      <c r="B11" s="67" t="inlineStr">
+        <is>
+          <t>Urgency (retargeting)</t>
+        </is>
+      </c>
+      <c r="C11" s="66" t="inlineStr">
+        <is>
+          <t>Seats are filling for Tuesday's live cloud bill teardown. Send your bill question, and if it's picked, we tear it down live (anonymised).</t>
+        </is>
+      </c>
+      <c r="D11" s="66" t="inlineStr">
+        <is>
+          <t>Last chance: free bill teardown</t>
+        </is>
+      </c>
+      <c r="E11" s="66" t="inlineStr">
+        <is>
+          <t>Tue 27 Oct · 4 PM IST</t>
+        </is>
+      </c>
+      <c r="F11" s="66" t="inlineStr">
+        <is>
+          <t>Sign up</t>
+        </is>
+      </c>
+      <c r="G11" s="66" t="inlineStr">
+        <is>
+          <t>V10, S5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="69" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="63" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>Angle</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="inlineStr">
+        <is>
+          <t>Intro text (keep under 150 characters)</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="E14" s="63" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
+      <c r="F14" s="63" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+      <c r="G14" s="63" t="inlineStr">
+        <is>
+          <t>Headline chars</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="67" t="inlineStr">
+        <is>
+          <t>L-A</t>
+        </is>
+      </c>
+      <c r="B15" s="67" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="C15" s="66" t="inlineStr">
+        <is>
+          <t>29% of cloud spend is wasted. Here's where it hides in Kubernetes and AI workloads. Free live session, 27 Oct.</t>
+        </is>
+      </c>
+      <c r="D15" s="66" t="inlineStr">
+        <is>
+          <t>AI Is Eating Your Cloud Bill: Free Live Session</t>
+        </is>
+      </c>
+      <c r="E15" s="66" t="inlineStr">
+        <is>
+          <t>Lead Gen Form + S2</t>
+        </is>
+      </c>
+      <c r="F15" s="66" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="G15" s="90">
+        <f>LEN(D15)</f>
+        <v>47.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="67" t="inlineStr">
+        <is>
+          <t>L-B</t>
+        </is>
+      </c>
+      <c r="B16" s="67" t="inlineStr">
+        <is>
+          <t>Teardown</t>
+        </is>
+      </c>
+      <c r="C16" s="66" t="inlineStr">
+        <is>
+          <t>Send us your cloud bill question. Our CTO will tear down 3 real (anonymised) bills live on 27 Oct.</t>
+        </is>
+      </c>
+      <c r="D16" s="66" t="inlineStr">
+        <is>
+          <t>Live Cloud Bill Teardown for SRE &amp; DevOps Teams</t>
+        </is>
+      </c>
+      <c r="E16" s="66" t="inlineStr">
+        <is>
+          <t>Lead Gen Form + S3</t>
+        </is>
+      </c>
+      <c r="F16" s="66" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="G16" s="90">
+        <f>LEN(D16)</f>
+        <v>47.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="67" t="inlineStr">
+        <is>
+          <t>L-C</t>
+        </is>
+      </c>
+      <c r="B17" s="67" t="inlineStr">
+        <is>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="C17" s="66" t="inlineStr">
+        <is>
+          <t>Free 27-point Cost Leak Checklist for Kubernetes, storage, data transfer and GPUs. Instant access when you register.</t>
+        </is>
+      </c>
+      <c r="D17" s="66" t="inlineStr">
+        <is>
+          <t>Get the 27-Point Cloud Cost Leak Checklist</t>
+        </is>
+      </c>
+      <c r="E17" s="66" t="inlineStr">
+        <is>
+          <t>Document ad L1</t>
+        </is>
+      </c>
+      <c r="F17" s="66" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="G17" s="90">
+        <f>LEN(D17)</f>
+        <v>42.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>L-D</t>
+        </is>
+      </c>
+      <c r="B18" s="67" t="inlineStr">
+        <is>
+          <t>Thought Leader (CTO post)</t>
+        </is>
+      </c>
+      <c r="C18" s="66" t="inlineStr">
+        <is>
+          <t>I review cloud bills every week. The same 5 leaks show up almost every time. I'm walking through all 5 live on 27 Oct.</t>
+        </is>
+      </c>
+      <c r="D18" s="66" t="inlineStr">
+        <is>
+          <t>Join my free session on cloud cost leaks</t>
+        </is>
+      </c>
+      <c r="E18" s="66" t="inlineStr">
+        <is>
+          <t>CTO's own post, promoted</t>
+        </is>
+      </c>
+      <c r="F18" s="66" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="G18" s="90">
+        <f>LEN(D18)</f>
+        <v>40.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="69" t="inlineStr">
+        <is>
+          <t>Google Search: ad groups and keywords</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="63" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>Ad group</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>Keywords ("phrase", [exact])</t>
+        </is>
+      </c>
+      <c r="D21" s="63" t="inlineStr"/>
+      <c r="E21" s="63" t="inlineStr"/>
+      <c r="F21" s="63" t="inlineStr"/>
+      <c r="G21" s="63" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="67" t="inlineStr">
+        <is>
+          <t>Kubernetes cost</t>
+        </is>
+      </c>
+      <c r="C22" s="66" t="inlineStr">
+        <is>
+          <t>"kubernetes cost optimization", "reduce kubernetes cost", [kubernetes cost management], "eks cost optimization", "aks cost optimization"</t>
+        </is>
+      </c>
+      <c r="D22" s="64" t="n"/>
+      <c r="E22" s="64" t="n"/>
+      <c r="F22" s="64" t="n"/>
+      <c r="G22" s="65" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="67" t="inlineStr">
+        <is>
+          <t>Cloud cost / FinOps</t>
+        </is>
+      </c>
+      <c r="C23" s="66" t="inlineStr">
+        <is>
+          <t>"cloud cost optimization", "reduce aws bill", "aws cost optimization", "finops for ai", "gpu cost optimization"</t>
+        </is>
+      </c>
+      <c r="D23" s="64" t="n"/>
+      <c r="E23" s="64" t="n"/>
+      <c r="F23" s="64" t="n"/>
+      <c r="G23" s="65" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" s="67" t="inlineStr">
+        <is>
+          <t>DevOps / SRE</t>
+        </is>
+      </c>
+      <c r="C24" s="66" t="inlineStr">
+        <is>
+          <t>"devops webinar", "sre webinar", "platform engineering webinar", "devops best practices 2026"</t>
+        </is>
+      </c>
+      <c r="D24" s="64" t="n"/>
+      <c r="E24" s="64" t="n"/>
+      <c r="F24" s="64" t="n"/>
+      <c r="G24" s="65" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="67" t="inlineStr"/>
+      <c r="B25" s="67" t="inlineStr">
+        <is>
+          <t>Negative keywords</t>
+        </is>
+      </c>
+      <c r="C25" s="66" t="inlineStr">
+        <is>
+          <t>jobs, job, salary, hiring, course, certification, training, institute, interview, internship, tutorial pdf, free download, udemy, coursera, fresher</t>
+        </is>
+      </c>
+      <c r="D25" s="64" t="n"/>
+      <c r="E25" s="64" t="n"/>
+      <c r="F25" s="64" t="n"/>
+      <c r="G25" s="65" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="69" t="inlineStr">
+        <is>
+          <t>Google Search: responsive search ad (shared by all 3 ad groups; put the ad-group keyword in headline 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="63" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D28" s="63" t="inlineStr">
+        <is>
+          <t>Chars</t>
+        </is>
+      </c>
+      <c r="E28" s="63" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="F28" s="63" t="inlineStr">
+        <is>
+          <t>OK?</t>
+        </is>
+      </c>
+      <c r="G28" s="63" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C29" s="66" t="inlineStr">
+        <is>
+          <t>Cut Kubernetes Costs</t>
+        </is>
+      </c>
+      <c r="D29" s="90">
+        <f>LEN(C29)</f>
+        <v>20.0</v>
+      </c>
+      <c r="E29" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F29" s="66" t="str">
+        <f>IF(D29&lt;=E29,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="66" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C30" s="66" t="inlineStr">
+        <is>
+          <t>Free Live CTO Session</t>
+        </is>
+      </c>
+      <c r="D30" s="90">
+        <f>LEN(C30)</f>
+        <v>21.0</v>
+      </c>
+      <c r="E30" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F30" s="66" t="str">
+        <f>IF(D30&lt;=E30,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="66" t="n">
+        <v>3</v>
+      </c>
+      <c r="B31" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C31" s="66" t="inlineStr">
+        <is>
+          <t>AI Is Eating Your Cloud Bill</t>
+        </is>
+      </c>
+      <c r="D31" s="90">
+        <f>LEN(C31)</f>
+        <v>28.0</v>
+      </c>
+      <c r="E31" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F31" s="66" t="str">
+        <f>IF(D31&lt;=E31,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="66" t="n">
+        <v>4</v>
+      </c>
+      <c r="B32" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C32" s="66" t="inlineStr">
+        <is>
+          <t>Live Cloud Bill Teardown</t>
+        </is>
+      </c>
+      <c r="D32" s="90">
+        <f>LEN(C32)</f>
+        <v>24.0</v>
+      </c>
+      <c r="E32" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F32" s="66" t="str">
+        <f>IF(D32&lt;=E32,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="66" t="n">
+        <v>5</v>
+      </c>
+      <c r="B33" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C33" s="66" t="inlineStr">
+        <is>
+          <t>For SRE &amp; DevOps Engineers</t>
+        </is>
+      </c>
+      <c r="D33" s="90">
+        <f>LEN(C33)</f>
+        <v>26.0</v>
+      </c>
+      <c r="E33" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F33" s="66" t="str">
+        <f>IF(D33&lt;=E33,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="66" t="n">
+        <v>6</v>
+      </c>
+      <c r="B34" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C34" s="66" t="inlineStr">
+        <is>
+          <t>29% of Cloud Spend Is Wasted</t>
+        </is>
+      </c>
+      <c r="D34" s="90">
+        <f>LEN(C34)</f>
+        <v>28.0</v>
+      </c>
+      <c r="E34" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F34" s="66" t="str">
+        <f>IF(D34&lt;=E34,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="66" t="n">
+        <v>7</v>
+      </c>
+      <c r="B35" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C35" s="66" t="inlineStr">
+        <is>
+          <t>Find 5 Hidden Cost Leaks</t>
+        </is>
+      </c>
+      <c r="D35" s="90">
+        <f>LEN(C35)</f>
+        <v>24.0</v>
+      </c>
+      <c r="E35" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F35" s="66" t="str">
+        <f>IF(D35&lt;=E35,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="66" t="n">
+        <v>8</v>
+      </c>
+      <c r="B36" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C36" s="66" t="inlineStr">
+        <is>
+          <t>Free 27-Point Checklist</t>
+        </is>
+      </c>
+      <c r="D36" s="90">
+        <f>LEN(C36)</f>
+        <v>23.0</v>
+      </c>
+      <c r="E36" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F36" s="66" t="str">
+        <f>IF(D36&lt;=E36,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="66" t="n">
+        <v>9</v>
+      </c>
+      <c r="B37" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C37" s="66" t="inlineStr">
+        <is>
+          <t>Tue 27 Oct, 4 PM IST</t>
+        </is>
+      </c>
+      <c r="D37" s="90">
+        <f>LEN(C37)</f>
+        <v>20.0</v>
+      </c>
+      <c r="E37" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F37" s="66" t="str">
+        <f>IF(D37&lt;=E37,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="66" t="n">
+        <v>10</v>
+      </c>
+      <c r="B38" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C38" s="66" t="inlineStr">
+        <is>
+          <t>No Sales Pitch, No Demo</t>
+        </is>
+      </c>
+      <c r="D38" s="90">
+        <f>LEN(C38)</f>
+        <v>23.0</v>
+      </c>
+      <c r="E38" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F38" s="66" t="str">
+        <f>IF(D38&lt;=E38,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="66" t="n">
+        <v>11</v>
+      </c>
+      <c r="B39" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C39" s="66" t="inlineStr">
+        <is>
+          <t>Ex-Microsoft CTO Explains</t>
+        </is>
+      </c>
+      <c r="D39" s="90">
+        <f>LEN(C39)</f>
+        <v>25.0</v>
+      </c>
+      <c r="E39" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F39" s="66" t="str">
+        <f>IF(D39&lt;=E39,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="66" t="n">
+        <v>12</v>
+      </c>
+      <c r="B40" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C40" s="66" t="inlineStr">
+        <is>
+          <t>Cut GPU &amp; AI Costs</t>
+        </is>
+      </c>
+      <c r="D40" s="90">
+        <f>LEN(C40)</f>
+        <v>18.0</v>
+      </c>
+      <c r="E40" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F40" s="66" t="str">
+        <f>IF(D40&lt;=E40,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="66" t="n">
+        <v>13</v>
+      </c>
+      <c r="B41" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C41" s="66" t="inlineStr">
+        <is>
+          <t>Rightsize Pods the Easy Way</t>
+        </is>
+      </c>
+      <c r="D41" s="90">
+        <f>LEN(C41)</f>
+        <v>27.0</v>
+      </c>
+      <c r="E41" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F41" s="66" t="str">
+        <f>IF(D41&lt;=E41,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="66" t="n">
+        <v>14</v>
+      </c>
+      <c r="B42" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C42" s="66" t="inlineStr">
+        <is>
+          <t>45 Minutes, Free</t>
+        </is>
+      </c>
+      <c r="D42" s="90">
+        <f>LEN(C42)</f>
+        <v>16.0</v>
+      </c>
+      <c r="E42" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F42" s="66" t="str">
+        <f>IF(D42&lt;=E42,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="66" t="n">
+        <v>15</v>
+      </c>
+      <c r="B43" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C43" s="66" t="inlineStr">
+        <is>
+          <t>Register Free Today</t>
+        </is>
+      </c>
+      <c r="D43" s="90">
+        <f>LEN(C43)</f>
+        <v>19.0</v>
+      </c>
+      <c r="E43" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="F43" s="66" t="str">
+        <f>IF(D43&lt;=E43,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="67" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C44" s="66" t="inlineStr">
+        <is>
+          <t>See where cloud money leaks in Kubernetes and AI workloads, and how to fix it this sprint.</t>
+        </is>
+      </c>
+      <c r="D44" s="90">
+        <f>LEN(C44)</f>
+        <v>90.0</v>
+      </c>
+      <c r="E44" s="90" t="n">
+        <v>90</v>
+      </c>
+      <c r="F44" s="66" t="str">
+        <f>IF(D44&lt;=E44,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="66" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="67" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C45" s="66" t="inlineStr">
+        <is>
+          <t>Free 45-min session for SRE, DevOps and cloud engineers. Real cloud bills torn down live.</t>
+        </is>
+      </c>
+      <c r="D45" s="90">
+        <f>LEN(C45)</f>
+        <v>89.0</v>
+      </c>
+      <c r="E45" s="90" t="n">
+        <v>90</v>
+      </c>
+      <c r="F45" s="66" t="str">
+        <f>IF(D45&lt;=E45,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="66" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" s="67" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C46" s="66" t="inlineStr">
+        <is>
+          <t>Register free and get the 27-point Cloud &amp; Kubernetes Cost Leak Checklist instantly.</t>
+        </is>
+      </c>
+      <c r="D46" s="90">
+        <f>LEN(C46)</f>
+        <v>84.0</v>
+      </c>
+      <c r="E46" s="90" t="n">
+        <v>90</v>
+      </c>
+      <c r="F46" s="66" t="str">
+        <f>IF(D46&lt;=E46,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="66" t="n">
+        <v>4</v>
+      </c>
+      <c r="B47" s="67" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C47" s="66" t="inlineStr">
+        <is>
+          <t>Join live for the full playbook, a certificate and a chance to win ₹5,000 vouchers.</t>
+        </is>
+      </c>
+      <c r="D47" s="90">
+        <f>LEN(C47)</f>
+        <v>83.0</v>
+      </c>
+      <c r="E47" s="90" t="n">
+        <v>90</v>
+      </c>
+      <c r="F47" s="66" t="str">
+        <f>IF(D47&lt;=E47,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="66" t="inlineStr"/>
+      <c r="B48" s="67" t="inlineStr">
+        <is>
+          <t>Sitelinks</t>
+        </is>
+      </c>
+      <c r="C48" s="66" t="inlineStr">
+        <is>
+          <t>Agenda · Speakers · Free Checklist · Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="69" t="inlineStr">
+        <is>
+          <t>Google Demand Gen</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="63" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B51" s="63" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C51" s="63" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="D51" s="63" t="inlineStr">
+        <is>
+          <t>Chars</t>
+        </is>
+      </c>
+      <c r="E51" s="63" t="inlineStr">
+        <is>
+          <t>Limit</t>
+        </is>
+      </c>
+      <c r="F51" s="63" t="inlineStr">
+        <is>
+          <t>OK?</t>
+        </is>
+      </c>
+      <c r="G51" s="63" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="B52" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C52" s="66" t="inlineStr">
+        <is>
+          <t>AI Is Eating Your Cloud Bill</t>
+        </is>
+      </c>
+      <c r="D52" s="90">
+        <f>LEN(C52)</f>
+        <v>28.0</v>
+      </c>
+      <c r="E52" s="90" t="n">
+        <v>40</v>
+      </c>
+      <c r="F52" s="66" t="str">
+        <f>IF(D52&lt;=E52,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="66" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C53" s="66" t="inlineStr">
+        <is>
+          <t>Find the 29% Your Cloud Wastes</t>
+        </is>
+      </c>
+      <c r="D53" s="90">
+        <f>LEN(C53)</f>
+        <v>30.0</v>
+      </c>
+      <c r="E53" s="90" t="n">
+        <v>40</v>
+      </c>
+      <c r="F53" s="66" t="str">
+        <f>IF(D53&lt;=E53,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="66" t="n">
+        <v>3</v>
+      </c>
+      <c r="B54" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C54" s="66" t="inlineStr">
+        <is>
+          <t>Free Live Cloud Bill Teardown</t>
+        </is>
+      </c>
+      <c r="D54" s="90">
+        <f>LEN(C54)</f>
+        <v>29.0</v>
+      </c>
+      <c r="E54" s="90" t="n">
+        <v>40</v>
+      </c>
+      <c r="F54" s="66" t="str">
+        <f>IF(D54&lt;=E54,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="66" t="n">
+        <v>4</v>
+      </c>
+      <c r="B55" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C55" s="66" t="inlineStr">
+        <is>
+          <t>5 Kubernetes Cost Leaks, Fixed</t>
+        </is>
+      </c>
+      <c r="D55" s="90">
+        <f>LEN(C55)</f>
+        <v>30.0</v>
+      </c>
+      <c r="E55" s="90" t="n">
+        <v>40</v>
+      </c>
+      <c r="F55" s="66" t="str">
+        <f>IF(D55&lt;=E55,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="66" t="n">
+        <v>5</v>
+      </c>
+      <c r="B56" s="67" t="inlineStr">
+        <is>
+          <t>Headline</t>
+        </is>
+      </c>
+      <c r="C56" s="66" t="inlineStr">
+        <is>
+          <t>Free CTO Session for Engineers</t>
+        </is>
+      </c>
+      <c r="D56" s="90">
+        <f>LEN(C56)</f>
+        <v>30.0</v>
+      </c>
+      <c r="E56" s="90" t="n">
+        <v>40</v>
+      </c>
+      <c r="F56" s="66" t="str">
+        <f>IF(D56&lt;=E56,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="B57" s="67" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C57" s="66" t="inlineStr">
+        <is>
+          <t>29% of cloud spend is wasted. See where it hides in Kubernetes and AI. Free, 27 Oct.</t>
+        </is>
+      </c>
+      <c r="D57" s="90">
+        <f>LEN(C57)</f>
+        <v>84.0</v>
+      </c>
+      <c r="E57" s="90" t="n">
+        <v>90</v>
+      </c>
+      <c r="F57" s="66" t="str">
+        <f>IF(D57&lt;=E57,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="66" t="n">
+        <v>2</v>
+      </c>
+      <c r="B58" s="67" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C58" s="66" t="inlineStr">
+        <is>
+          <t>Free 27-point Cost Leak Checklist when you register. Live session Tue 27 Oct, 4 PM IST.</t>
+        </is>
+      </c>
+      <c r="D58" s="90">
+        <f>LEN(C58)</f>
+        <v>87.0</v>
+      </c>
+      <c r="E58" s="90" t="n">
+        <v>90</v>
+      </c>
+      <c r="F58" s="66" t="str">
+        <f>IF(D58&lt;=E58,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="66" t="n">
+        <v>3</v>
+      </c>
+      <c r="B59" s="67" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C59" s="66" t="inlineStr">
+        <is>
+          <t>For SRE, DevOps and cloud engineers. 45 min, no sales pitch, real bills torn down live.</t>
+        </is>
+      </c>
+      <c r="D59" s="90">
+        <f>LEN(C59)</f>
+        <v>87.0</v>
+      </c>
+      <c r="E59" s="90" t="n">
+        <v>90</v>
+      </c>
+      <c r="F59" s="66" t="str">
+        <f>IF(D59&lt;=E59,"OK","Too long")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="74" t="inlineStr">
+        <is>
+          <t>Rules for every ad: speaker face in the first second, the date in the ad, 'Free' visible, no Zarthi product claims, the 29% figure always credited to State of FinOps 2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="C23:G23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2977,7 +4401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3527,7 +4951,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5072,7 +6496,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5476,7 +6900,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6223,7 +7647,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7055,7 +8479,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF262626"/>
@@ -7454,7 +8878,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFB42A"/>
@@ -7859,7 +9283,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF262626"/>
@@ -11056,6 +12480,1275 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Audience universe: how many people we can reach on Meta, LinkedIn and Google</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="75" t="inlineStr">
+        <is>
+          <t>Cream = estimate you can edit. Blue = paste the real number from each ad tool on setup day (Meta Ads Manager 'Estimated audience size', LinkedIn Campaign Manager 'Forecasted results', Google Keyword Planner).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="75" t="inlineStr">
+        <is>
+          <t>Exact audience sizes only exist inside each platform's ad tool; the numbers below are bottom-up estimates from public data, to be replaced on setup day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="127" t="inlineStr">
+        <is>
+          <t>A. The real market in India (people, not platform accounts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="63" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B6" s="63" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="inlineStr"/>
+      <c r="F6" s="63" t="inlineStr"/>
+      <c r="G6" s="63" t="inlineStr">
+        <is>
+          <t>Source / logic</t>
+        </is>
+      </c>
+      <c r="H6" s="63" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>Indian developers on GitHub</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="inlineStr">
+        <is>
+          <t>All developer accounts (includes students and inactive)</t>
+        </is>
+      </c>
+      <c r="C7" s="82" t="n">
+        <v>21900000</v>
+      </c>
+      <c r="D7" s="82" t="n">
+        <v>21900000</v>
+      </c>
+      <c r="E7" s="66" t="inlineStr"/>
+      <c r="F7" s="66" t="inlineStr"/>
+      <c r="G7" s="66" t="inlineStr">
+        <is>
+          <t>GitHub Octoverse 2025: India #2 with 21.9M developers</t>
+        </is>
+      </c>
+      <c r="H7" s="68" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="67" t="inlineStr">
+        <is>
+          <t>Indian tech industry workforce</t>
+        </is>
+      </c>
+      <c r="B8" s="66" t="inlineStr">
+        <is>
+          <t>People employed in the Indian tech industry</t>
+        </is>
+      </c>
+      <c r="C8" s="82" t="n">
+        <v>5800000</v>
+      </c>
+      <c r="D8" s="82" t="n">
+        <v>5800000</v>
+      </c>
+      <c r="E8" s="66" t="inlineStr"/>
+      <c r="F8" s="66" t="inlineStr"/>
+      <c r="G8" s="66" t="inlineStr">
+        <is>
+          <t>NASSCOM: tech workforce 5.8M in FY2025</t>
+        </is>
+      </c>
+      <c r="H8" s="68" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="67" t="inlineStr">
+        <is>
+          <t>Our target roles (SRE, DevOps, cloud, platform, backend devs on cloud)</t>
+        </is>
+      </c>
+      <c r="B9" s="66" t="inlineStr">
+        <is>
+          <t>Inside and outside IT companies (GCCs, startups, enterprises)</t>
+        </is>
+      </c>
+      <c r="C9" s="82" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="D9" s="82" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="E9" s="66" t="inlineStr"/>
+      <c r="F9" s="66" t="inlineStr"/>
+      <c r="G9" s="66" t="inlineStr">
+        <is>
+          <t>Estimate: ~25–40% of the tech workforce works on cloud infrastructure or backend services</t>
+        </is>
+      </c>
+      <c r="H9" s="66" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="67" t="inlineStr">
+        <is>
+          <t>With 3–15 years of experience</t>
+        </is>
+      </c>
+      <c r="B10" s="66" t="inlineStr">
+        <is>
+          <t>Removes freshers and very senior people</t>
+        </is>
+      </c>
+      <c r="C10" s="78">
+        <f>ROUND(C9*0.55,-4)</f>
+        <v>830000.0</v>
+      </c>
+      <c r="D10" s="78">
+        <f>ROUND(D9*0.65,-4)</f>
+        <v>1620000.0</v>
+      </c>
+      <c r="E10" s="66" t="inlineStr"/>
+      <c r="F10" s="66" t="inlineStr"/>
+      <c r="G10" s="66" t="inlineStr">
+        <is>
+          <t>Estimate: 55–65% of the target roles</t>
+        </is>
+      </c>
+      <c r="H10" s="66" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="67" t="inlineStr">
+        <is>
+          <t>In our cities (6 metros + tier-2)</t>
+        </is>
+      </c>
+      <c r="B11" s="66" t="inlineStr">
+        <is>
+          <t>Bengaluru, Hyderabad, Pune, Delhi-NCR, Chennai, Mumbai + tier-2</t>
+        </is>
+      </c>
+      <c r="C11" s="78">
+        <f>ROUND(C10*0.75,-4)</f>
+        <v>620000.0</v>
+      </c>
+      <c r="D11" s="78">
+        <f>ROUND(D10*0.85,-4)</f>
+        <v>1380000.0</v>
+      </c>
+      <c r="E11" s="66" t="inlineStr"/>
+      <c r="F11" s="66" t="inlineStr"/>
+      <c r="G11" s="66" t="inlineStr">
+        <is>
+          <t>Estimate: 75–85% of these jobs are in these cities</t>
+        </is>
+      </c>
+      <c r="H11" s="66" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="84" t="inlineStr">
+        <is>
+          <t>Core target audience (real people)</t>
+        </is>
+      </c>
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>The people we actually want in the webinar</t>
+        </is>
+      </c>
+      <c r="C12" s="85">
+        <f>C11</f>
+        <v>620000.0</v>
+      </c>
+      <c r="D12" s="85">
+        <f>D11</f>
+        <v>1380000.0</v>
+      </c>
+      <c r="E12" s="87" t="inlineStr"/>
+      <c r="F12" s="87" t="inlineStr"/>
+      <c r="G12" s="84" t="str">
+        <f>"We need "&amp;TEXT(Funnel!B8,"#,##0")&amp;" registrations = "&amp;TEXT(Funnel!B8/C12,"0.00%")&amp;" of the low estimate"</f>
+        <v>We need 880 registrations = 0.14% of the low estimate</v>
+      </c>
+      <c r="H12" s="87" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="127" t="inlineStr">
+        <is>
+          <t>B. Universe by platform and ad set</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="63" t="inlineStr">
+        <is>
+          <t>Platform / ad set</t>
+        </is>
+      </c>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>Targeting used</t>
+        </is>
+      </c>
+      <c r="C15" s="63" t="inlineStr">
+        <is>
+          <t>Est. universe (low)</t>
+        </is>
+      </c>
+      <c r="D15" s="63" t="inlineStr">
+        <is>
+          <t>Est. universe (high)</t>
+        </is>
+      </c>
+      <c r="E15" s="63" t="inlineStr">
+        <is>
+          <t>Actual (from ad tool)</t>
+        </is>
+      </c>
+      <c r="F15" s="63" t="inlineStr">
+        <is>
+          <t>Impressions needed (plan)</t>
+        </is>
+      </c>
+      <c r="G15" s="63" t="inlineStr">
+        <is>
+          <t>How estimated</t>
+        </is>
+      </c>
+      <c r="H15" s="63" t="inlineStr">
+        <is>
+          <t>Times each person must see an ad*</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="67" t="inlineStr">
+        <is>
+          <t>Meta: total India ad reach</t>
+        </is>
+      </c>
+      <c r="B16" s="66" t="inlineStr">
+        <is>
+          <t>Facebook 403M + Instagram 481M ad reach (overlap)</t>
+        </is>
+      </c>
+      <c r="C16" s="82" t="n">
+        <v>450000000</v>
+      </c>
+      <c r="D16" s="82" t="n">
+        <v>600000000</v>
+      </c>
+      <c r="E16" s="128" t="n"/>
+      <c r="F16" s="66" t="inlineStr"/>
+      <c r="G16" s="66" t="inlineStr">
+        <is>
+          <t>DataReportal / Meta ad tools, late 2025</t>
+        </is>
+      </c>
+      <c r="H16" s="66" t="inlineStr"/>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="67" t="inlineStr">
+        <is>
+          <t>Meta M1: cloud &amp; DevOps interests</t>
+        </is>
+      </c>
+      <c r="B17" s="66" t="inlineStr">
+        <is>
+          <t>Age 24–45, 6 metros + tier-2; interests AWS, Azure, GCP, DevOps, Kubernetes, Docker, Terraform, SRE, Linux</t>
+        </is>
+      </c>
+      <c r="C17" s="82" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="D17" s="82" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="E17" s="128" t="n"/>
+      <c r="F17" s="78">
+        <f>ROUND((Budget!B4+Budget!B5)/Funnel!$B$9/Funnel!$B$11,-3)</f>
+        <v>711000.0</v>
+      </c>
+      <c r="G17" s="66" t="inlineStr">
+        <is>
+          <t>Estimate: interest audiences include students and enthusiasts, so they're far bigger than the real target</t>
+        </is>
+      </c>
+      <c r="H17" s="129">
+        <f>IFERROR(F17/(C17+C18),0)</f>
+        <v>0.0395</v>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>Meta M2: developer interests</t>
+        </is>
+      </c>
+      <c r="B18" s="66" t="inlineStr">
+        <is>
+          <t>Same geo/age; GitHub, Stack Overflow, software development, Python, Java, Go, microservices</t>
+        </is>
+      </c>
+      <c r="C18" s="82" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="D18" s="82" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="E18" s="128" t="n"/>
+      <c r="F18" s="66" t="inlineStr"/>
+      <c r="G18" s="66" t="inlineStr">
+        <is>
+          <t>Estimate, excluding M1</t>
+        </is>
+      </c>
+      <c r="H18" s="66" t="inlineStr"/>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="67" t="inlineStr">
+        <is>
+          <t>Meta: real target people reachable</t>
+        </is>
+      </c>
+      <c r="B19" s="66" t="inlineStr">
+        <is>
+          <t>Core target (row 12) who use Facebook or Instagram</t>
+        </is>
+      </c>
+      <c r="C19" s="78">
+        <f>ROUND(C12*0.7,-4)</f>
+        <v>430000.0</v>
+      </c>
+      <c r="D19" s="78">
+        <f>ROUND(D12*0.85,-4)</f>
+        <v>1170000.0</v>
+      </c>
+      <c r="E19" s="128" t="n"/>
+      <c r="F19" s="66" t="inlineStr"/>
+      <c r="G19" s="66" t="inlineStr">
+        <is>
+          <t>Estimate: 70–85% of the core target use FB/IG</t>
+        </is>
+      </c>
+      <c r="H19" s="66" t="inlineStr"/>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="67" t="inlineStr">
+        <is>
+          <t>LinkedIn: total India members</t>
+        </is>
+      </c>
+      <c r="B20" s="66" t="inlineStr">
+        <is>
+          <t>All members</t>
+        </is>
+      </c>
+      <c r="C20" s="82" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="D20" s="82" t="n">
+        <v>167000000</v>
+      </c>
+      <c r="E20" s="128" t="n"/>
+      <c r="F20" s="66" t="inlineStr"/>
+      <c r="G20" s="66" t="inlineStr">
+        <is>
+          <t>LinkedIn India membership 2026 (several trackers)</t>
+        </is>
+      </c>
+      <c r="H20" s="66" t="inlineStr"/>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>LinkedIn L1: job titles + 3–15 yrs + company 51+</t>
+        </is>
+      </c>
+      <c r="B21" s="66" t="inlineStr">
+        <is>
+          <t>DevOps Engineer/Lead, SRE, Cloud Engineer, Platform Engineer, Cloud Architect, Engineering Manager; India</t>
+        </is>
+      </c>
+      <c r="C21" s="82" t="n">
+        <v>600000</v>
+      </c>
+      <c r="D21" s="82" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E21" s="128" t="n"/>
+      <c r="F21" s="78">
+        <f>ROUND(Budget!B6/Funnel!$B$9/Funnel!$B$11,-3)</f>
+        <v>67000.0</v>
+      </c>
+      <c r="G21" s="66" t="inlineStr">
+        <is>
+          <t>Estimate from title counts; LinkedIn shows the exact size when the audience is built</t>
+        </is>
+      </c>
+      <c r="H21" s="129">
+        <f>IFERROR(F21/C22,0)</f>
+        <v>0.319047619047619</v>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="67" t="inlineStr">
+        <is>
+          <t>LinkedIn: active in our 18-day window</t>
+        </is>
+      </c>
+      <c r="B22" s="66" t="inlineStr">
+        <is>
+          <t>Members who log in during the campaign</t>
+        </is>
+      </c>
+      <c r="C22" s="78">
+        <f>ROUND(C21*0.35,-4)</f>
+        <v>210000.0</v>
+      </c>
+      <c r="D22" s="78">
+        <f>ROUND(D21*0.45,-4)</f>
+        <v>450000.0</v>
+      </c>
+      <c r="E22" s="128" t="n"/>
+      <c r="F22" s="66" t="inlineStr"/>
+      <c r="G22" s="66" t="inlineStr">
+        <is>
+          <t>Estimate: 35–45% log in during any 3-week window</t>
+        </is>
+      </c>
+      <c r="H22" s="66" t="inlineStr"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="67" t="inlineStr">
+        <is>
+          <t>Google Demand Gen: custom segments</t>
+        </is>
+      </c>
+      <c r="B23" s="66" t="inlineStr">
+        <is>
+          <t>People who searched Kubernetes, DevOps, Terraform, AWS cost, FinOps, SRE (YouTube, Discover, Gmail)</t>
+        </is>
+      </c>
+      <c r="C23" s="82" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D23" s="82" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="E23" s="128" t="n"/>
+      <c r="F23" s="78">
+        <f>ROUND(Budget!B8/Funnel!$B$9/Funnel!$B$11,-3)</f>
+        <v>111000.0</v>
+      </c>
+      <c r="G23" s="66" t="inlineStr">
+        <is>
+          <t>Estimate from ~170k monthly searches on these terms (table C) plus YouTube viewing signals</t>
+        </is>
+      </c>
+      <c r="H23" s="129">
+        <f>IFERROR(F23/C23,0)</f>
+        <v>0.111</v>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="67" t="inlineStr">
+        <is>
+          <t>Google Search: high-intent cost searches</t>
+        </is>
+      </c>
+      <c r="B24" s="66" t="inlineStr">
+        <is>
+          <t>Searches per month in India for cost keywords (table C)</t>
+        </is>
+      </c>
+      <c r="C24" s="78">
+        <f>C44</f>
+        <v>5890.0</v>
+      </c>
+      <c r="D24" s="78">
+        <f>C44</f>
+        <v>5890.0</v>
+      </c>
+      <c r="E24" s="128" t="n"/>
+      <c r="F24" s="66" t="inlineStr"/>
+      <c r="G24" s="66" t="inlineStr">
+        <is>
+          <t>Ahrefs keyword data, India; this is searches per month, not people</t>
+        </is>
+      </c>
+      <c r="H24" s="66" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="75" t="inlineStr">
+        <is>
+          <t>*Impressions needed ÷ low-end universe. Below 3 = plenty of room; above 6 = the audience will tire and costs rise. Google Search is checked separately in table D.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="127" t="inlineStr">
+        <is>
+          <t>C. Google Search volume in India (Ahrefs, monthly searches, last 12 months)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="63" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>Intent</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>Monthly searches</t>
+        </is>
+      </c>
+      <c r="D28" s="63" t="inlineStr">
+        <is>
+          <t>CPC (US$)</t>
+        </is>
+      </c>
+      <c r="E28" s="63" t="inlineStr">
+        <is>
+          <t>Use?</t>
+        </is>
+      </c>
+      <c r="F28" s="63" t="inlineStr"/>
+      <c r="G28" s="63" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="H28" s="63" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="67" t="inlineStr">
+        <is>
+          <t>finops</t>
+        </is>
+      </c>
+      <c r="B29" s="66" t="inlineStr">
+        <is>
+          <t>Cost (mixed: also certification seekers)</t>
+        </is>
+      </c>
+      <c r="C29" s="78" t="n">
+        <v>2800</v>
+      </c>
+      <c r="D29" s="129" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E29" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F29" s="66" t="inlineStr"/>
+      <c r="G29" s="66" t="inlineStr"/>
+      <c r="H29" s="66" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="67" t="inlineStr">
+        <is>
+          <t>aws cost explorer</t>
+        </is>
+      </c>
+      <c r="B30" s="66" t="inlineStr">
+        <is>
+          <t>Cost: existing AWS users</t>
+        </is>
+      </c>
+      <c r="C30" s="78" t="n">
+        <v>800</v>
+      </c>
+      <c r="D30" s="129" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F30" s="66" t="inlineStr"/>
+      <c r="G30" s="66" t="inlineStr">
+        <is>
+          <t>Best intent: people already looking at their bill</t>
+        </is>
+      </c>
+      <c r="H30" s="66" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="67" t="inlineStr">
+        <is>
+          <t>kubecost</t>
+        </is>
+      </c>
+      <c r="B31" s="66" t="inlineStr">
+        <is>
+          <t>Cost: Kubernetes cost tool</t>
+        </is>
+      </c>
+      <c r="C31" s="78" t="n">
+        <v>500</v>
+      </c>
+      <c r="D31" s="129" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E31" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F31" s="66" t="inlineStr"/>
+      <c r="G31" s="66" t="inlineStr"/>
+      <c r="H31" s="66" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="67" t="inlineStr">
+        <is>
+          <t>cloud cost optimization</t>
+        </is>
+      </c>
+      <c r="B32" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C32" s="78" t="n">
+        <v>450</v>
+      </c>
+      <c r="D32" s="129" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E32" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F32" s="66" t="inlineStr"/>
+      <c r="G32" s="66" t="inlineStr"/>
+      <c r="H32" s="66" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="67" t="inlineStr">
+        <is>
+          <t>aws cost optimization</t>
+        </is>
+      </c>
+      <c r="B33" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C33" s="78" t="n">
+        <v>300</v>
+      </c>
+      <c r="D33" s="129" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E33" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F33" s="66" t="inlineStr"/>
+      <c r="G33" s="66" t="inlineStr"/>
+      <c r="H33" s="66" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="67" t="inlineStr">
+        <is>
+          <t>cloud cost management</t>
+        </is>
+      </c>
+      <c r="B34" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C34" s="78" t="n">
+        <v>250</v>
+      </c>
+      <c r="D34" s="129" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E34" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F34" s="66" t="inlineStr"/>
+      <c r="G34" s="66" t="inlineStr"/>
+      <c r="H34" s="66" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="67" t="inlineStr">
+        <is>
+          <t>azure cost management</t>
+        </is>
+      </c>
+      <c r="B35" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C35" s="78" t="n">
+        <v>250</v>
+      </c>
+      <c r="D35" s="129" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E35" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F35" s="66" t="inlineStr"/>
+      <c r="G35" s="66" t="inlineStr"/>
+      <c r="H35" s="66" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="67" t="inlineStr">
+        <is>
+          <t>cloud cost</t>
+        </is>
+      </c>
+      <c r="B36" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C36" s="78" t="n">
+        <v>150</v>
+      </c>
+      <c r="D36" s="129" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E36" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F36" s="66" t="inlineStr"/>
+      <c r="G36" s="66" t="inlineStr"/>
+      <c r="H36" s="66" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="67" t="inlineStr">
+        <is>
+          <t>finops for ai</t>
+        </is>
+      </c>
+      <c r="B37" s="66" t="inlineStr">
+        <is>
+          <t>Cost / AI</t>
+        </is>
+      </c>
+      <c r="C37" s="78" t="n">
+        <v>100</v>
+      </c>
+      <c r="D37" s="129" t="n"/>
+      <c r="E37" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F37" s="66" t="inlineStr"/>
+      <c r="G37" s="66" t="inlineStr"/>
+      <c r="H37" s="66" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="67" t="inlineStr">
+        <is>
+          <t>devops best practices</t>
+        </is>
+      </c>
+      <c r="B38" s="66" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="C38" s="78" t="n">
+        <v>100</v>
+      </c>
+      <c r="D38" s="129" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E38" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F38" s="66" t="inlineStr"/>
+      <c r="G38" s="66" t="inlineStr"/>
+      <c r="H38" s="66" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="67" t="inlineStr">
+        <is>
+          <t>kubernetes cost optimization</t>
+        </is>
+      </c>
+      <c r="B39" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C39" s="78" t="n">
+        <v>80</v>
+      </c>
+      <c r="D39" s="129" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E39" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F39" s="66" t="inlineStr"/>
+      <c r="G39" s="66" t="inlineStr"/>
+      <c r="H39" s="66" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="67" t="inlineStr">
+        <is>
+          <t>kubernetes cost management</t>
+        </is>
+      </c>
+      <c r="B40" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C40" s="78" t="n">
+        <v>50</v>
+      </c>
+      <c r="D40" s="129" t="n"/>
+      <c r="E40" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F40" s="66" t="inlineStr"/>
+      <c r="G40" s="66" t="inlineStr"/>
+      <c r="H40" s="66" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="67" t="inlineStr">
+        <is>
+          <t>eks cost optimization</t>
+        </is>
+      </c>
+      <c r="B41" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C41" s="78" t="n">
+        <v>30</v>
+      </c>
+      <c r="D41" s="129" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="E41" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F41" s="66" t="inlineStr"/>
+      <c r="G41" s="66" t="inlineStr"/>
+      <c r="H41" s="66" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="67" t="inlineStr">
+        <is>
+          <t>aks cost optimization</t>
+        </is>
+      </c>
+      <c r="B42" s="66" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C42" s="78" t="n">
+        <v>30</v>
+      </c>
+      <c r="D42" s="129" t="n"/>
+      <c r="E42" s="66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F42" s="66" t="inlineStr"/>
+      <c r="G42" s="66" t="inlineStr"/>
+      <c r="H42" s="66" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="67" t="inlineStr">
+        <is>
+          <t>Not used (too broad or learners)</t>
+        </is>
+      </c>
+      <c r="B43" s="66" t="inlineStr">
+        <is>
+          <t>devops 77,000 · kubernetes 55,000 · terraform 30,000 · aws devops 1,800 · platform engineering 1,400 · SRE 900 · finops certification 450 · devops webinar 10</t>
+        </is>
+      </c>
+      <c r="C43" s="64" t="n"/>
+      <c r="D43" s="64" t="n"/>
+      <c r="E43" s="64" t="n"/>
+      <c r="F43" s="64" t="n"/>
+      <c r="G43" s="64" t="n"/>
+      <c r="H43" s="65" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="84" t="inlineStr">
+        <is>
+          <t>Total high-intent searches per month</t>
+        </is>
+      </c>
+      <c r="B44" s="87" t="inlineStr"/>
+      <c r="C44" s="85">
+        <f>SUM(C29:C42)</f>
+        <v>5890.0</v>
+      </c>
+      <c r="D44" s="87" t="inlineStr"/>
+      <c r="E44" s="87" t="inlineStr"/>
+      <c r="F44" s="87" t="inlineStr"/>
+      <c r="G44" s="87" t="inlineStr"/>
+      <c r="H44" s="87" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="127" t="inlineStr">
+        <is>
+          <t>D. Can Google Search deliver what the plan asks? (capacity check)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="63" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B47" s="63" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C47" s="63" t="inlineStr"/>
+      <c r="D47" s="63" t="inlineStr"/>
+      <c r="E47" s="63" t="inlineStr"/>
+      <c r="F47" s="63" t="inlineStr"/>
+      <c r="G47" s="63" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="H47" s="63" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="67" t="inlineStr">
+        <is>
+          <t>High-intent searches per month</t>
+        </is>
+      </c>
+      <c r="B48" s="78">
+        <f>C44</f>
+        <v>5890.0</v>
+      </c>
+      <c r="C48" s="66" t="inlineStr"/>
+      <c r="D48" s="66" t="inlineStr"/>
+      <c r="E48" s="66" t="inlineStr"/>
+      <c r="F48" s="66" t="inlineStr"/>
+      <c r="G48" s="66" t="inlineStr">
+        <is>
+          <t>Table C</t>
+        </is>
+      </c>
+      <c r="H48" s="66" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="67" t="inlineStr">
+        <is>
+          <t>Days of ads</t>
+        </is>
+      </c>
+      <c r="B49" s="90">
+        <f>Budget!D30</f>
+        <v>18.0</v>
+      </c>
+      <c r="C49" s="66" t="inlineStr"/>
+      <c r="D49" s="66" t="inlineStr"/>
+      <c r="E49" s="66" t="inlineStr"/>
+      <c r="F49" s="66" t="inlineStr"/>
+      <c r="G49" s="66" t="inlineStr">
+        <is>
+          <t>Budget tab</t>
+        </is>
+      </c>
+      <c r="H49" s="66" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="67" t="inlineStr">
+        <is>
+          <t>Searches during the campaign</t>
+        </is>
+      </c>
+      <c r="B50" s="78">
+        <f>ROUND(B48*B49/30,0)</f>
+        <v>3534.0</v>
+      </c>
+      <c r="C50" s="66" t="inlineStr"/>
+      <c r="D50" s="66" t="inlineStr"/>
+      <c r="E50" s="66" t="inlineStr"/>
+      <c r="F50" s="66" t="inlineStr"/>
+      <c r="G50" s="66" t="inlineStr"/>
+      <c r="H50" s="66" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="67" t="inlineStr">
+        <is>
+          <t>Share of searches our ad shows on</t>
+        </is>
+      </c>
+      <c r="B51" s="77" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C51" s="66" t="inlineStr"/>
+      <c r="D51" s="66" t="inlineStr"/>
+      <c r="E51" s="66" t="inlineStr"/>
+      <c r="F51" s="66" t="inlineStr"/>
+      <c r="G51" s="66" t="inlineStr">
+        <is>
+          <t>Estimate with a competitive bid</t>
+        </is>
+      </c>
+      <c r="H51" s="66" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="67" t="inlineStr">
+        <is>
+          <t>Ad click-through rate</t>
+        </is>
+      </c>
+      <c r="B52" s="77" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C52" s="66" t="inlineStr"/>
+      <c r="D52" s="66" t="inlineStr"/>
+      <c r="E52" s="66" t="inlineStr"/>
+      <c r="F52" s="66" t="inlineStr"/>
+      <c r="G52" s="66" t="inlineStr">
+        <is>
+          <t>Typical for search ads</t>
+        </is>
+      </c>
+      <c r="H52" s="66" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="67" t="inlineStr">
+        <is>
+          <t>Landing page conversion</t>
+        </is>
+      </c>
+      <c r="B53" s="98">
+        <f>Funnel!B9</f>
+        <v>0.15</v>
+      </c>
+      <c r="C53" s="66" t="inlineStr"/>
+      <c r="D53" s="66" t="inlineStr"/>
+      <c r="E53" s="66" t="inlineStr"/>
+      <c r="F53" s="66" t="inlineStr"/>
+      <c r="G53" s="66" t="inlineStr">
+        <is>
+          <t>Funnel tab</t>
+        </is>
+      </c>
+      <c r="H53" s="66" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="67" t="inlineStr">
+        <is>
+          <t>Registrations Search can realistically deliver</t>
+        </is>
+      </c>
+      <c r="B54" s="100">
+        <f>ROUND(B50*B51*B52*B53,0)</f>
+        <v>16.0</v>
+      </c>
+      <c r="C54" s="66" t="inlineStr"/>
+      <c r="D54" s="66" t="inlineStr"/>
+      <c r="E54" s="66" t="inlineStr"/>
+      <c r="F54" s="66" t="inlineStr"/>
+      <c r="G54" s="66" t="inlineStr"/>
+      <c r="H54" s="66" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="67" t="inlineStr">
+        <is>
+          <t>Registrations the plan expects from Search</t>
+        </is>
+      </c>
+      <c r="B55" s="100">
+        <f>Budget!B7</f>
+        <v>80.0</v>
+      </c>
+      <c r="C55" s="66" t="inlineStr"/>
+      <c r="D55" s="66" t="inlineStr"/>
+      <c r="E55" s="66" t="inlineStr"/>
+      <c r="F55" s="66" t="inlineStr"/>
+      <c r="G55" s="66" t="inlineStr">
+        <is>
+          <t>Budget tab</t>
+        </is>
+      </c>
+      <c r="H55" s="66" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="130" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B56" s="130" t="str">
+        <f>IF(B55&gt;B54,"Over capacity: move "&amp;(B55-B54)&amp;" registrations from Search to Demand Gen or Meta","OK")</f>
+        <v>Over capacity: move 64 registrations from Search to Demand Gen or Meta</v>
+      </c>
+      <c r="C56" s="64" t="n"/>
+      <c r="D56" s="64" t="n"/>
+      <c r="E56" s="64" t="n"/>
+      <c r="F56" s="64" t="n"/>
+      <c r="G56" s="64" t="n"/>
+      <c r="H56" s="65" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="127" t="inlineStr">
+        <is>
+          <t>E. What this means</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="131" t="inlineStr">
+        <is>
+          <t>1. The market is big enough: we need ~880 registrations from about 0.6–1.4 million real target people, under 0.15% of them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="131" t="inlineStr">
+        <is>
+          <t>2. Meta has the most room, but its interest audiences are 10–20× bigger than the real target, so creative and the form must filter out students and job seekers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="131" t="inlineStr">
+        <is>
+          <t>3. LinkedIn is the most precise (real job titles) but small and expensive; 60 registrations barely touch it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="131" t="inlineStr">
+        <is>
+          <t>4. Google Search is the tightest: only ~6,000 high-intent cost searches a month in India. Treat it as a small, high-quality source and move the rest to Demand Gen or Meta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="131" t="inlineStr">
+        <is>
+          <t>5. On setup day, paste the real sizes from each ad tool into the blue column and check the 'times each person must see an ad' column stays below 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="75" t="inlineStr">
+        <is>
+          <t>Sources: GitHub Octoverse 2025; NASSCOM FY2025 strategic review; DataReportal (Meta ad reach, India, late 2025); LinkedIn India membership trackers 2026; Ahrefs Keywords Explorer (India).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B43:H43"/>
+    <mergeCell ref="B56:H56"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FF262626"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -11556,7 +14249,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFB42A"/>
@@ -12710,7 +15403,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13287,7 +15980,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13996,1406 +16689,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:G61"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="62" t="inlineStr">
-        <is>
-          <t>Ad copy: Meta, LinkedIn and Google</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="74" t="inlineStr">
-        <is>
-          <t>Character counts are formulas so you can edit and check. Limits: Google headline 30, description 90; Demand Gen headline 40; LinkedIn headline 70.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="69" t="inlineStr">
-        <is>
-          <t>Meta (Facebook + Instagram)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="63" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B5" s="63" t="inlineStr">
-        <is>
-          <t>Angle</t>
-        </is>
-      </c>
-      <c r="C5" s="63" t="inlineStr">
-        <is>
-          <t>Primary text</t>
-        </is>
-      </c>
-      <c r="D5" s="63" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="E5" s="63" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="F5" s="63" t="inlineStr">
-        <is>
-          <t>Button</t>
-        </is>
-      </c>
-      <c r="G5" s="63" t="inlineStr">
-        <is>
-          <t>Use with</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="67" t="inlineStr">
-        <is>
-          <t>M-A</t>
-        </is>
-      </c>
-      <c r="B6" s="67" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="C6" s="66" t="inlineStr">
-        <is>
-          <t>29% of cloud spend is wasted, and it's rising again (State of FinOps 2026). On 27 Oct our CTO shows the 5 places it leaks in Kubernetes and AI workloads, with a live bill teardown. Free checklist when you register.</t>
-        </is>
-      </c>
-      <c r="D6" s="66" t="inlineStr">
-        <is>
-          <t>Find the 29% your cloud bill wastes</t>
-        </is>
-      </c>
-      <c r="E6" s="66" t="inlineStr">
-        <is>
-          <t>Free live session · 27 Oct · 4 PM IST</t>
-        </is>
-      </c>
-      <c r="F6" s="66" t="inlineStr">
-        <is>
-          <t>Sign up</t>
-        </is>
-      </c>
-      <c r="G6" s="66" t="inlineStr">
-        <is>
-          <t>V2, S2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="67" t="inlineStr">
-        <is>
-          <t>M-B</t>
-        </is>
-      </c>
-      <c r="B7" s="67" t="inlineStr">
-        <is>
-          <t>Pain</t>
-        </is>
-      </c>
-      <c r="C7" s="66" t="inlineStr">
-        <is>
-          <t>Bill up. Traffic flat. And somehow it's the DevOps team's problem. Learn how SREs find idle clusters, oversized pods and idle GPUs, and fix them this sprint.</t>
-        </is>
-      </c>
-      <c r="D7" s="66" t="inlineStr">
-        <is>
-          <t>Your cloud bill went up again?</t>
-        </is>
-      </c>
-      <c r="E7" s="66" t="inlineStr">
-        <is>
-          <t>45 min · Free · No sales pitch</t>
-        </is>
-      </c>
-      <c r="F7" s="66" t="inlineStr">
-        <is>
-          <t>Sign up</t>
-        </is>
-      </c>
-      <c r="G7" s="66" t="inlineStr">
-        <is>
-          <t>V3, S1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="67" t="inlineStr">
-        <is>
-          <t>M-C</t>
-        </is>
-      </c>
-      <c r="B8" s="67" t="inlineStr">
-        <is>
-          <t>Curiosity</t>
-        </is>
-      </c>
-      <c r="C8" s="66" t="inlineStr">
-        <is>
-          <t>3 places your Kubernetes bill leaks. Number 2 surprises almost everyone. Our CTO (ex-Microsoft, 15 yrs) covers all 5 live on 27 Oct.</t>
-        </is>
-      </c>
-      <c r="D8" s="66" t="inlineStr">
-        <is>
-          <t>3 Kubernetes bill leaks (no. 2!)</t>
-        </is>
-      </c>
-      <c r="E8" s="66" t="inlineStr">
-        <is>
-          <t>Free CTO session for engineers</t>
-        </is>
-      </c>
-      <c r="F8" s="66" t="inlineStr">
-        <is>
-          <t>Learn more</t>
-        </is>
-      </c>
-      <c r="G8" s="66" t="inlineStr">
-        <is>
-          <t>V3, C1</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="67" t="inlineStr">
-        <is>
-          <t>M-D</t>
-        </is>
-      </c>
-      <c r="B9" s="67" t="inlineStr">
-        <is>
-          <t>Offer</t>
-        </is>
-      </c>
-      <c r="C9" s="66" t="inlineStr">
-        <is>
-          <t>Register free and get our 27-point Cloud &amp; Kubernetes Cost Leak Checklist right away. Join live on 27 Oct for the full playbook, a certificate and a ₹5,000 lucky draw.</t>
-        </is>
-      </c>
-      <c r="D9" s="66" t="inlineStr">
-        <is>
-          <t>Free 27-point Cost Leak Checklist</t>
-        </is>
-      </c>
-      <c r="E9" s="66" t="inlineStr">
-        <is>
-          <t>Instant download when you register</t>
-        </is>
-      </c>
-      <c r="F9" s="66" t="inlineStr">
-        <is>
-          <t>Download</t>
-        </is>
-      </c>
-      <c r="G9" s="66" t="inlineStr">
-        <is>
-          <t>S4, V1</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="67" t="inlineStr">
-        <is>
-          <t>M-E</t>
-        </is>
-      </c>
-      <c r="B10" s="67" t="inlineStr">
-        <is>
-          <t>Career</t>
-        </is>
-      </c>
-      <c r="C10" s="66" t="inlineStr">
-        <is>
-          <t>The engineers who get promoted fastest can explain the cloud bill. Learn how a CTO reads one, live on 27 Oct. For SRE, DevOps, cloud and platform engineers.</t>
-        </is>
-      </c>
-      <c r="D10" s="66" t="inlineStr">
-        <is>
-          <t>Explain the bill. Get the promotion.</t>
-        </is>
-      </c>
-      <c r="E10" s="66" t="inlineStr">
-        <is>
-          <t>Think Like a CTO · Episode 1</t>
-        </is>
-      </c>
-      <c r="F10" s="66" t="inlineStr">
-        <is>
-          <t>Sign up</t>
-        </is>
-      </c>
-      <c r="G10" s="66" t="inlineStr">
-        <is>
-          <t>V4, C3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="67" t="inlineStr">
-        <is>
-          <t>M-F</t>
-        </is>
-      </c>
-      <c r="B11" s="67" t="inlineStr">
-        <is>
-          <t>Urgency (retargeting)</t>
-        </is>
-      </c>
-      <c r="C11" s="66" t="inlineStr">
-        <is>
-          <t>Seats are filling for Tuesday's live cloud bill teardown. Send your bill question, and if it's picked, we tear it down live (anonymised).</t>
-        </is>
-      </c>
-      <c r="D11" s="66" t="inlineStr">
-        <is>
-          <t>Last chance: free bill teardown</t>
-        </is>
-      </c>
-      <c r="E11" s="66" t="inlineStr">
-        <is>
-          <t>Tue 27 Oct · 4 PM IST</t>
-        </is>
-      </c>
-      <c r="F11" s="66" t="inlineStr">
-        <is>
-          <t>Sign up</t>
-        </is>
-      </c>
-      <c r="G11" s="66" t="inlineStr">
-        <is>
-          <t>V10, S5</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="69" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="63" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B14" s="63" t="inlineStr">
-        <is>
-          <t>Angle</t>
-        </is>
-      </c>
-      <c r="C14" s="63" t="inlineStr">
-        <is>
-          <t>Intro text (keep under 150 characters)</t>
-        </is>
-      </c>
-      <c r="D14" s="63" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="E14" s="63" t="inlineStr">
-        <is>
-          <t>Format</t>
-        </is>
-      </c>
-      <c r="F14" s="63" t="inlineStr">
-        <is>
-          <t>Button</t>
-        </is>
-      </c>
-      <c r="G14" s="63" t="inlineStr">
-        <is>
-          <t>Headline chars</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="67" t="inlineStr">
-        <is>
-          <t>L-A</t>
-        </is>
-      </c>
-      <c r="B15" s="67" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="C15" s="66" t="inlineStr">
-        <is>
-          <t>29% of cloud spend is wasted. Here's where it hides in Kubernetes and AI workloads. Free live session, 27 Oct.</t>
-        </is>
-      </c>
-      <c r="D15" s="66" t="inlineStr">
-        <is>
-          <t>AI Is Eating Your Cloud Bill: Free Live Session</t>
-        </is>
-      </c>
-      <c r="E15" s="66" t="inlineStr">
-        <is>
-          <t>Lead Gen Form + S2</t>
-        </is>
-      </c>
-      <c r="F15" s="66" t="inlineStr">
-        <is>
-          <t>Register</t>
-        </is>
-      </c>
-      <c r="G15" s="90">
-        <f>LEN(D15)</f>
-        <v>47.0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="67" t="inlineStr">
-        <is>
-          <t>L-B</t>
-        </is>
-      </c>
-      <c r="B16" s="67" t="inlineStr">
-        <is>
-          <t>Teardown</t>
-        </is>
-      </c>
-      <c r="C16" s="66" t="inlineStr">
-        <is>
-          <t>Send us your cloud bill question. Our CTO will tear down 3 real (anonymised) bills live on 27 Oct.</t>
-        </is>
-      </c>
-      <c r="D16" s="66" t="inlineStr">
-        <is>
-          <t>Live Cloud Bill Teardown for SRE &amp; DevOps Teams</t>
-        </is>
-      </c>
-      <c r="E16" s="66" t="inlineStr">
-        <is>
-          <t>Lead Gen Form + S3</t>
-        </is>
-      </c>
-      <c r="F16" s="66" t="inlineStr">
-        <is>
-          <t>Register</t>
-        </is>
-      </c>
-      <c r="G16" s="90">
-        <f>LEN(D16)</f>
-        <v>47.0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="67" t="inlineStr">
-        <is>
-          <t>L-C</t>
-        </is>
-      </c>
-      <c r="B17" s="67" t="inlineStr">
-        <is>
-          <t>Checklist</t>
-        </is>
-      </c>
-      <c r="C17" s="66" t="inlineStr">
-        <is>
-          <t>Free 27-point Cost Leak Checklist for Kubernetes, storage, data transfer and GPUs. Instant access when you register.</t>
-        </is>
-      </c>
-      <c r="D17" s="66" t="inlineStr">
-        <is>
-          <t>Get the 27-Point Cloud Cost Leak Checklist</t>
-        </is>
-      </c>
-      <c r="E17" s="66" t="inlineStr">
-        <is>
-          <t>Document ad L1</t>
-        </is>
-      </c>
-      <c r="F17" s="66" t="inlineStr">
-        <is>
-          <t>Download</t>
-        </is>
-      </c>
-      <c r="G17" s="90">
-        <f>LEN(D17)</f>
-        <v>42.0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="67" t="inlineStr">
-        <is>
-          <t>L-D</t>
-        </is>
-      </c>
-      <c r="B18" s="67" t="inlineStr">
-        <is>
-          <t>Thought Leader (CTO post)</t>
-        </is>
-      </c>
-      <c r="C18" s="66" t="inlineStr">
-        <is>
-          <t>I review cloud bills every week. The same 5 leaks show up almost every time. I'm walking through all 5 live on 27 Oct.</t>
-        </is>
-      </c>
-      <c r="D18" s="66" t="inlineStr">
-        <is>
-          <t>Join my free session on cloud cost leaks</t>
-        </is>
-      </c>
-      <c r="E18" s="66" t="inlineStr">
-        <is>
-          <t>CTO's own post, promoted</t>
-        </is>
-      </c>
-      <c r="F18" s="66" t="inlineStr">
-        <is>
-          <t>Register</t>
-        </is>
-      </c>
-      <c r="G18" s="90">
-        <f>LEN(D18)</f>
-        <v>40.0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="69" t="inlineStr">
-        <is>
-          <t>Google Search: ad groups and keywords</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="63" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B21" s="63" t="inlineStr">
-        <is>
-          <t>Ad group</t>
-        </is>
-      </c>
-      <c r="C21" s="63" t="inlineStr">
-        <is>
-          <t>Keywords ("phrase", [exact])</t>
-        </is>
-      </c>
-      <c r="D21" s="63" t="inlineStr"/>
-      <c r="E21" s="63" t="inlineStr"/>
-      <c r="F21" s="63" t="inlineStr"/>
-      <c r="G21" s="63" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="67" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" s="67" t="inlineStr">
-        <is>
-          <t>Kubernetes cost</t>
-        </is>
-      </c>
-      <c r="C22" s="66" t="inlineStr">
-        <is>
-          <t>"kubernetes cost optimization", "reduce kubernetes cost", [kubernetes cost management], "eks cost optimization", "aks cost optimization"</t>
-        </is>
-      </c>
-      <c r="D22" s="64" t="n"/>
-      <c r="E22" s="64" t="n"/>
-      <c r="F22" s="64" t="n"/>
-      <c r="G22" s="65" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="67" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" s="67" t="inlineStr">
-        <is>
-          <t>Cloud cost / FinOps</t>
-        </is>
-      </c>
-      <c r="C23" s="66" t="inlineStr">
-        <is>
-          <t>"cloud cost optimization", "reduce aws bill", "aws cost optimization", "finops for ai", "gpu cost optimization"</t>
-        </is>
-      </c>
-      <c r="D23" s="64" t="n"/>
-      <c r="E23" s="64" t="n"/>
-      <c r="F23" s="64" t="n"/>
-      <c r="G23" s="65" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="67" t="n">
-        <v>3</v>
-      </c>
-      <c r="B24" s="67" t="inlineStr">
-        <is>
-          <t>DevOps / SRE</t>
-        </is>
-      </c>
-      <c r="C24" s="66" t="inlineStr">
-        <is>
-          <t>"devops webinar", "sre webinar", "platform engineering webinar", "devops best practices 2026"</t>
-        </is>
-      </c>
-      <c r="D24" s="64" t="n"/>
-      <c r="E24" s="64" t="n"/>
-      <c r="F24" s="64" t="n"/>
-      <c r="G24" s="65" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="67" t="inlineStr"/>
-      <c r="B25" s="67" t="inlineStr">
-        <is>
-          <t>Negative keywords</t>
-        </is>
-      </c>
-      <c r="C25" s="66" t="inlineStr">
-        <is>
-          <t>jobs, job, salary, hiring, course, certification, training, institute, interview, internship, tutorial pdf, free download, udemy, coursera, fresher</t>
-        </is>
-      </c>
-      <c r="D25" s="64" t="n"/>
-      <c r="E25" s="64" t="n"/>
-      <c r="F25" s="64" t="n"/>
-      <c r="G25" s="65" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="69" t="inlineStr">
-        <is>
-          <t>Google Search: responsive search ad (shared by all 3 ad groups; put the ad-group keyword in headline 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="63" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B28" s="63" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C28" s="63" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="D28" s="63" t="inlineStr">
-        <is>
-          <t>Chars</t>
-        </is>
-      </c>
-      <c r="E28" s="63" t="inlineStr">
-        <is>
-          <t>Limit</t>
-        </is>
-      </c>
-      <c r="F28" s="63" t="inlineStr">
-        <is>
-          <t>OK?</t>
-        </is>
-      </c>
-      <c r="G28" s="63" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="66" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C29" s="66" t="inlineStr">
-        <is>
-          <t>Cut Kubernetes Costs</t>
-        </is>
-      </c>
-      <c r="D29" s="90">
-        <f>LEN(C29)</f>
-        <v>20.0</v>
-      </c>
-      <c r="E29" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F29" s="66" t="str">
-        <f>IF(D29&lt;=E29,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="66" t="n">
-        <v>2</v>
-      </c>
-      <c r="B30" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C30" s="66" t="inlineStr">
-        <is>
-          <t>Free Live CTO Session</t>
-        </is>
-      </c>
-      <c r="D30" s="90">
-        <f>LEN(C30)</f>
-        <v>21.0</v>
-      </c>
-      <c r="E30" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F30" s="66" t="str">
-        <f>IF(D30&lt;=E30,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="66" t="n">
-        <v>3</v>
-      </c>
-      <c r="B31" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C31" s="66" t="inlineStr">
-        <is>
-          <t>AI Is Eating Your Cloud Bill</t>
-        </is>
-      </c>
-      <c r="D31" s="90">
-        <f>LEN(C31)</f>
-        <v>28.0</v>
-      </c>
-      <c r="E31" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F31" s="66" t="str">
-        <f>IF(D31&lt;=E31,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="66" t="n">
-        <v>4</v>
-      </c>
-      <c r="B32" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C32" s="66" t="inlineStr">
-        <is>
-          <t>Live Cloud Bill Teardown</t>
-        </is>
-      </c>
-      <c r="D32" s="90">
-        <f>LEN(C32)</f>
-        <v>24.0</v>
-      </c>
-      <c r="E32" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F32" s="66" t="str">
-        <f>IF(D32&lt;=E32,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="66" t="n">
-        <v>5</v>
-      </c>
-      <c r="B33" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C33" s="66" t="inlineStr">
-        <is>
-          <t>For SRE &amp; DevOps Engineers</t>
-        </is>
-      </c>
-      <c r="D33" s="90">
-        <f>LEN(C33)</f>
-        <v>26.0</v>
-      </c>
-      <c r="E33" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F33" s="66" t="str">
-        <f>IF(D33&lt;=E33,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="66" t="n">
-        <v>6</v>
-      </c>
-      <c r="B34" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C34" s="66" t="inlineStr">
-        <is>
-          <t>29% of Cloud Spend Is Wasted</t>
-        </is>
-      </c>
-      <c r="D34" s="90">
-        <f>LEN(C34)</f>
-        <v>28.0</v>
-      </c>
-      <c r="E34" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F34" s="66" t="str">
-        <f>IF(D34&lt;=E34,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="66" t="n">
-        <v>7</v>
-      </c>
-      <c r="B35" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C35" s="66" t="inlineStr">
-        <is>
-          <t>Find 5 Hidden Cost Leaks</t>
-        </is>
-      </c>
-      <c r="D35" s="90">
-        <f>LEN(C35)</f>
-        <v>24.0</v>
-      </c>
-      <c r="E35" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F35" s="66" t="str">
-        <f>IF(D35&lt;=E35,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="66" t="n">
-        <v>8</v>
-      </c>
-      <c r="B36" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C36" s="66" t="inlineStr">
-        <is>
-          <t>Free 27-Point Checklist</t>
-        </is>
-      </c>
-      <c r="D36" s="90">
-        <f>LEN(C36)</f>
-        <v>23.0</v>
-      </c>
-      <c r="E36" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F36" s="66" t="str">
-        <f>IF(D36&lt;=E36,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="66" t="n">
-        <v>9</v>
-      </c>
-      <c r="B37" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C37" s="66" t="inlineStr">
-        <is>
-          <t>Tue 27 Oct, 4 PM IST</t>
-        </is>
-      </c>
-      <c r="D37" s="90">
-        <f>LEN(C37)</f>
-        <v>20.0</v>
-      </c>
-      <c r="E37" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F37" s="66" t="str">
-        <f>IF(D37&lt;=E37,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="66" t="n">
-        <v>10</v>
-      </c>
-      <c r="B38" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C38" s="66" t="inlineStr">
-        <is>
-          <t>No Sales Pitch, No Demo</t>
-        </is>
-      </c>
-      <c r="D38" s="90">
-        <f>LEN(C38)</f>
-        <v>23.0</v>
-      </c>
-      <c r="E38" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F38" s="66" t="str">
-        <f>IF(D38&lt;=E38,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="66" t="n">
-        <v>11</v>
-      </c>
-      <c r="B39" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C39" s="66" t="inlineStr">
-        <is>
-          <t>Ex-Microsoft CTO Explains</t>
-        </is>
-      </c>
-      <c r="D39" s="90">
-        <f>LEN(C39)</f>
-        <v>25.0</v>
-      </c>
-      <c r="E39" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F39" s="66" t="str">
-        <f>IF(D39&lt;=E39,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="66" t="n">
-        <v>12</v>
-      </c>
-      <c r="B40" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C40" s="66" t="inlineStr">
-        <is>
-          <t>Cut GPU &amp; AI Costs</t>
-        </is>
-      </c>
-      <c r="D40" s="90">
-        <f>LEN(C40)</f>
-        <v>18.0</v>
-      </c>
-      <c r="E40" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F40" s="66" t="str">
-        <f>IF(D40&lt;=E40,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="66" t="n">
-        <v>13</v>
-      </c>
-      <c r="B41" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C41" s="66" t="inlineStr">
-        <is>
-          <t>Rightsize Pods the Easy Way</t>
-        </is>
-      </c>
-      <c r="D41" s="90">
-        <f>LEN(C41)</f>
-        <v>27.0</v>
-      </c>
-      <c r="E41" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F41" s="66" t="str">
-        <f>IF(D41&lt;=E41,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="66" t="n">
-        <v>14</v>
-      </c>
-      <c r="B42" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C42" s="66" t="inlineStr">
-        <is>
-          <t>45 Minutes, Free</t>
-        </is>
-      </c>
-      <c r="D42" s="90">
-        <f>LEN(C42)</f>
-        <v>16.0</v>
-      </c>
-      <c r="E42" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F42" s="66" t="str">
-        <f>IF(D42&lt;=E42,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="66" t="n">
-        <v>15</v>
-      </c>
-      <c r="B43" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C43" s="66" t="inlineStr">
-        <is>
-          <t>Register Free Today</t>
-        </is>
-      </c>
-      <c r="D43" s="90">
-        <f>LEN(C43)</f>
-        <v>19.0</v>
-      </c>
-      <c r="E43" s="90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F43" s="66" t="str">
-        <f>IF(D43&lt;=E43,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="66" t="n">
-        <v>1</v>
-      </c>
-      <c r="B44" s="67" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C44" s="66" t="inlineStr">
-        <is>
-          <t>See where cloud money leaks in Kubernetes and AI workloads, and how to fix it this sprint.</t>
-        </is>
-      </c>
-      <c r="D44" s="90">
-        <f>LEN(C44)</f>
-        <v>90.0</v>
-      </c>
-      <c r="E44" s="90" t="n">
-        <v>90</v>
-      </c>
-      <c r="F44" s="66" t="str">
-        <f>IF(D44&lt;=E44,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="66" t="n">
-        <v>2</v>
-      </c>
-      <c r="B45" s="67" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C45" s="66" t="inlineStr">
-        <is>
-          <t>Free 45-min session for SRE, DevOps and cloud engineers. Real cloud bills torn down live.</t>
-        </is>
-      </c>
-      <c r="D45" s="90">
-        <f>LEN(C45)</f>
-        <v>89.0</v>
-      </c>
-      <c r="E45" s="90" t="n">
-        <v>90</v>
-      </c>
-      <c r="F45" s="66" t="str">
-        <f>IF(D45&lt;=E45,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="66" t="n">
-        <v>3</v>
-      </c>
-      <c r="B46" s="67" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C46" s="66" t="inlineStr">
-        <is>
-          <t>Register free and get the 27-point Cloud &amp; Kubernetes Cost Leak Checklist instantly.</t>
-        </is>
-      </c>
-      <c r="D46" s="90">
-        <f>LEN(C46)</f>
-        <v>84.0</v>
-      </c>
-      <c r="E46" s="90" t="n">
-        <v>90</v>
-      </c>
-      <c r="F46" s="66" t="str">
-        <f>IF(D46&lt;=E46,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="66" t="n">
-        <v>4</v>
-      </c>
-      <c r="B47" s="67" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C47" s="66" t="inlineStr">
-        <is>
-          <t>Join live for the full playbook, a certificate and a chance to win ₹5,000 vouchers.</t>
-        </is>
-      </c>
-      <c r="D47" s="90">
-        <f>LEN(C47)</f>
-        <v>83.0</v>
-      </c>
-      <c r="E47" s="90" t="n">
-        <v>90</v>
-      </c>
-      <c r="F47" s="66" t="str">
-        <f>IF(D47&lt;=E47,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="66" t="inlineStr"/>
-      <c r="B48" s="67" t="inlineStr">
-        <is>
-          <t>Sitelinks</t>
-        </is>
-      </c>
-      <c r="C48" s="66" t="inlineStr">
-        <is>
-          <t>Agenda · Speakers · Free Checklist · Register</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="69" t="inlineStr">
-        <is>
-          <t>Google Demand Gen</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="63" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B51" s="63" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C51" s="63" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="D51" s="63" t="inlineStr">
-        <is>
-          <t>Chars</t>
-        </is>
-      </c>
-      <c r="E51" s="63" t="inlineStr">
-        <is>
-          <t>Limit</t>
-        </is>
-      </c>
-      <c r="F51" s="63" t="inlineStr">
-        <is>
-          <t>OK?</t>
-        </is>
-      </c>
-      <c r="G51" s="63" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="66" t="n">
-        <v>1</v>
-      </c>
-      <c r="B52" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C52" s="66" t="inlineStr">
-        <is>
-          <t>AI Is Eating Your Cloud Bill</t>
-        </is>
-      </c>
-      <c r="D52" s="90">
-        <f>LEN(C52)</f>
-        <v>28.0</v>
-      </c>
-      <c r="E52" s="90" t="n">
-        <v>40</v>
-      </c>
-      <c r="F52" s="66" t="str">
-        <f>IF(D52&lt;=E52,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="66" t="n">
-        <v>2</v>
-      </c>
-      <c r="B53" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C53" s="66" t="inlineStr">
-        <is>
-          <t>Find the 29% Your Cloud Wastes</t>
-        </is>
-      </c>
-      <c r="D53" s="90">
-        <f>LEN(C53)</f>
-        <v>30.0</v>
-      </c>
-      <c r="E53" s="90" t="n">
-        <v>40</v>
-      </c>
-      <c r="F53" s="66" t="str">
-        <f>IF(D53&lt;=E53,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="66" t="n">
-        <v>3</v>
-      </c>
-      <c r="B54" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C54" s="66" t="inlineStr">
-        <is>
-          <t>Free Live Cloud Bill Teardown</t>
-        </is>
-      </c>
-      <c r="D54" s="90">
-        <f>LEN(C54)</f>
-        <v>29.0</v>
-      </c>
-      <c r="E54" s="90" t="n">
-        <v>40</v>
-      </c>
-      <c r="F54" s="66" t="str">
-        <f>IF(D54&lt;=E54,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="66" t="n">
-        <v>4</v>
-      </c>
-      <c r="B55" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C55" s="66" t="inlineStr">
-        <is>
-          <t>5 Kubernetes Cost Leaks, Fixed</t>
-        </is>
-      </c>
-      <c r="D55" s="90">
-        <f>LEN(C55)</f>
-        <v>30.0</v>
-      </c>
-      <c r="E55" s="90" t="n">
-        <v>40</v>
-      </c>
-      <c r="F55" s="66" t="str">
-        <f>IF(D55&lt;=E55,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="66" t="n">
-        <v>5</v>
-      </c>
-      <c r="B56" s="67" t="inlineStr">
-        <is>
-          <t>Headline</t>
-        </is>
-      </c>
-      <c r="C56" s="66" t="inlineStr">
-        <is>
-          <t>Free CTO Session for Engineers</t>
-        </is>
-      </c>
-      <c r="D56" s="90">
-        <f>LEN(C56)</f>
-        <v>30.0</v>
-      </c>
-      <c r="E56" s="90" t="n">
-        <v>40</v>
-      </c>
-      <c r="F56" s="66" t="str">
-        <f>IF(D56&lt;=E56,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="66" t="n">
-        <v>1</v>
-      </c>
-      <c r="B57" s="67" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C57" s="66" t="inlineStr">
-        <is>
-          <t>29% of cloud spend is wasted. See where it hides in Kubernetes and AI. Free, 27 Oct.</t>
-        </is>
-      </c>
-      <c r="D57" s="90">
-        <f>LEN(C57)</f>
-        <v>84.0</v>
-      </c>
-      <c r="E57" s="90" t="n">
-        <v>90</v>
-      </c>
-      <c r="F57" s="66" t="str">
-        <f>IF(D57&lt;=E57,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="66" t="n">
-        <v>2</v>
-      </c>
-      <c r="B58" s="67" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C58" s="66" t="inlineStr">
-        <is>
-          <t>Free 27-point Cost Leak Checklist when you register. Live session Tue 27 Oct, 4 PM IST.</t>
-        </is>
-      </c>
-      <c r="D58" s="90">
-        <f>LEN(C58)</f>
-        <v>87.0</v>
-      </c>
-      <c r="E58" s="90" t="n">
-        <v>90</v>
-      </c>
-      <c r="F58" s="66" t="str">
-        <f>IF(D58&lt;=E58,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="66" t="n">
-        <v>3</v>
-      </c>
-      <c r="B59" s="67" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C59" s="66" t="inlineStr">
-        <is>
-          <t>For SRE, DevOps and cloud engineers. 45 min, no sales pitch, real bills torn down live.</t>
-        </is>
-      </c>
-      <c r="D59" s="90">
-        <f>LEN(C59)</f>
-        <v>87.0</v>
-      </c>
-      <c r="E59" s="90" t="n">
-        <v>90</v>
-      </c>
-      <c r="F59" s="66" t="str">
-        <f>IF(D59&lt;=E59,"OK","Too long")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="74" t="inlineStr">
-        <is>
-          <t>Rules for every ad: speaker face in the first second, the date in the ad, 'Free' visible, no Zarthi product claims, the 29% figure always credited to State of FinOps 2026.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="C23:G23"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>